<commit_message>
Realign the diagnostic to the real estate vertical and tighten mobile layouts
Question bank, findings, checklist, niches, modules, producer brief,
industries, labels, schemas, and docs now target commercial real estate
owners and multifamily owners/managers, with real estate branch
triggers (owned buildings, third-party manager, site vendors,
residential tenants, workforce, investors, environmental). FMCSA
enrichment is removed. Reporting question columns are renamed for the
new industries. The public header, producer header, dashboard stats,
assessment form footers, and lead page grid are adjusted so nothing
overflows at phone widths; verified with screenshots at 390px and 1280px.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JbEPs9eRjvDhvYpso2k2wq
</commit_message>
<xml_diff>
--- a/docs/marketready-question-bank.xlsx
+++ b/docs/marketready-question-bank.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from code on 2026-09-02T19:38:39.475Z. Regenerate with: npm run docs:bank</t>
+          <t>Generated from code on 2026-09-02T21:30:54.262Z. Regenerate with: npm run docs:bank</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -587,7 +587,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -675,12 +675,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>business changes 0; profile recent change true/false</t>
+          <t>business changes 0; profile recent acquisition true/false</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -692,22 +692,22 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>fleet_branch</t>
+          <t>management_agreement_branch</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>hasVehicles true; fleet controls 0</t>
+          <t>usesThirdPartyManager true; management agreement 0</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>branch applicable; critical flag br_fleet_controls</t>
+          <t>branch applicable; critical flag br_management_agreement</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>module=contracts; COI 0, requirements 1, subcontractor 1</t>
+          <t>module=contracts; COI 0, requirements 1, vendor transfer 1</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Who owns the insurance program, when renewal work begins, and how limits are decided.</t>
+          <t>Who owns the insurance program across the portfolio, when renewal work begins, and how limits and deductibles are decided.</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Data &amp; market readiness</t>
+          <t>Property data &amp; market readiness</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>How well exposure data and business changes are documented and presented to carriers.</t>
+          <t>How well the statement of values, acquisitions and dispositions, and building updates are documented and presented to carriers.</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Cyber, payment authorization, safety, and training practices that underwriters ask about.</t>
+          <t>Tenant and applicant data, rent and vendor payment controls, and property inspection and life-safety practices.</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>How incidents are reported, open claims are reviewed, and root causes are tracked.</t>
+          <t>How incidents at the properties are reported, open claims are reviewed, and corrective actions are tracked.</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Whether contracts, insurance requirements, and certificate verification work as one system.</t>
+          <t>Whether leases, vendor agreements, insurance requirements, and certificate verification work as one system.</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>How new locations, products, technology, and regulations are reviewed for risk impact.</t>
+          <t>How acquisitions, new property types, regulations, and new exposures like EV charging are reviewed for risk impact.</t>
         </is>
       </c>
     </row>
@@ -1006,88 +1006,88 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>3PL, warehousing &amp; distribution</t>
+          <t>Commercial real estate owner / investor</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>3PL / Warehousing</t>
+          <t>Commercial RE</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Third-party logistics, public and contract warehousing, cold chain, fulfillment, and regional distribution.</t>
+          <t>Office, industrial and flex, retail, mixed-use, and net-lease portfolios, whether self-managed or with a third-party manager.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>493110, 493120, 484110, 484121, 488510</t>
+          <t>531110, 531120, 531190, 531390</t>
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Carriers evaluating warehousing and 3PL accounts look closely at warehouse legal liability, cargo and customer contracts, fleet controls, fire protection, and how consistently incidents are reported.</t>
+          <t>Property underwriters price commercial portfolios on the quality of the statement of values, construction and protection data, roof and building-system updates, how carrier recommendations were handled, and how lease and vendor requirements transfer risk.</t>
         </is>
       </c>
       <c r="H2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="I2" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="4" t="n">
         <v>1.25</v>
       </c>
-      <c r="J2" s="4" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="L2" s="4" t="n">
-        <v>1.5</v>
-      </c>
       <c r="M2" s="4" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Light manufacturing</t>
+          <t>Multifamily owner / property manager</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Multifamily</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Fabrication, assembly, food and beverage, plastics, packaging, electronics, and other light industrial operations.</t>
+          <t>Apartment communities, student and workforce housing, and third-party residential management.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>332, 333, 335, 311, 326, 339</t>
+          <t>531110, 531311, 531390</t>
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Underwriters reviewing manufacturers focus on product liability and recall exposure, machine guarding and workers' compensation history, property valuation, business interruption, and supplier and customer contract terms.</t>
+          <t>Multifamily carriers look closely at habitability and life-safety practices, renters insurance enforcement, fair-housing training, vendor certificates for snow and ice and contractors, claim frequency, and how quickly incidents are reported.</t>
         </is>
       </c>
       <c r="H3" s="4" t="n">
@@ -1103,7 +1103,7 @@
         <v>1.25</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="M3" s="4" t="n">
         <v>1</v>
@@ -1117,26 +1117,30 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Other middle-market business</t>
+          <t>Other real estate operator</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Other RE</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Any other commercial operation. Uses generic weighting.</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr"/>
+          <t>Self-storage, hospitality assets, senior housing, associations, land, or a mixed portfolio. Uses generic weighting.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
       <c r="F4" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Carriers evaluate every account on the quality of its exposure data, controls, claims history, and the clarity of the story that accompanies the submission.</t>
+          <t>Carriers evaluate every real estate account on the quality of its property data, the controls at each location, claims history, and the clarity of the story that accompanies the submission.</t>
         </is>
       </c>
       <c r="H4" s="4" t="n">
@@ -1224,12 +1228,12 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>weight_logistics_3pl</t>
+          <t>weight_cre_owner</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>weight_light_manufacturing</t>
+          <t>weight_multifamily</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
@@ -1270,12 +1274,12 @@
       <c r="E2" s="4" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>When does renewal preparation typically begin relative to your policy expiration?</t>
+          <t>When does renewal preparation for the portfolio typically begin relative to policy expiration?</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Carriers reward complete submissions delivered early. Late starts compress negotiation time.</t>
+          <t>Property markets reward complete, early submissions. A late start means values and building updates never make it into the story carriers see.</t>
         </is>
       </c>
       <c r="H2" s="4" t="n">
@@ -1292,7 +1296,7 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Renewal preparation appears to begin inside 30 days of expiration, which limits the ability to document controls and approach alternative markets.</t>
+          <t>Renewal preparation appears to begin inside 30 days of expiration, which limits the ability to update values, document building improvements, and approach alternative markets.</t>
         </is>
       </c>
     </row>
@@ -1318,10 +1322,14 @@
       <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Who owns the insurance program internally, and how is that responsibility defined?</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
+          <t>Who owns the insurance program for the portfolio, and how is that responsibility defined?</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>In many real estate organizations this sits between ownership, an asset manager, a controller, and the property manager.</t>
+        </is>
+      </c>
       <c r="H3" s="4" t="n">
         <v>2</v>
       </c>
@@ -1350,18 +1358,18 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Limit rationale</t>
+          <t>Limit and deductible rationale</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>How are policy limits and deductibles decided each year?</t>
+          <t>How are liability limits, property deductibles, and umbrella limits decided each year?</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>This question asks about your decision process, not whether the limits are adequate.</t>
+          <t>This asks about your decision process, not whether the limits are adequate.</t>
         </is>
       </c>
       <c r="H4" s="4" t="n">
@@ -1392,16 +1400,20 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Exposure data</t>
+          <t>Statement of values</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>How are exposure values (payroll, revenue, property values, vehicle schedules, inventory) validated before submission?</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr"/>
+          <t>How is the statement of values (replacement cost, construction and protection details, occupancy, square footage, year built, updates) maintained and validated before submission?</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Replacement cost that is dictated by the insurer, or carried forward, is the most common reason a property submission is discounted.</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="n">
         <v>3</v>
       </c>
@@ -1430,13 +1442,13 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Business change documentation</t>
+          <t>Portfolio changes</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>How are operational changes (new services, locations, equipment, customers, headcount) communicated to your insurance program during the year?</t>
+          <t>How are acquisitions, dispositions, renovations, new leases, and occupancy changes communicated to your insurance program during the year?</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -1468,18 +1480,18 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Submission visibility</t>
+          <t>Your risk profile in the market</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>How much visibility do you have into what is actually sent to carriers about your company?</t>
+          <t>Do you know how your story is being told in the marketplace, and do you see what is sent to insurance companies about the portfolio?</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>The underwriting story is the narrative and evidence that accompanies applications and loss runs.</t>
+          <t>Brokers who never saw your environmental consultant's report, your capital plan, or your maintenance program cannot present them.</t>
         </is>
       </c>
       <c r="H7" s="4" t="n">
@@ -1510,21 +1522,25 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Cyber controls</t>
+          <t>Data security</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr"/>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Which of the following best describes your cyber controls (MFA, backups, endpoint protection, incident response)?</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr"/>
+          <t>What data do you hold on tenants, applicants, and investors, how is it stored and shared, and how is it protected?</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Applications, background checks, banking details, and investor reporting are all sensitive. Property-management software vendors should be part of the answer.</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>2</v>
@@ -1534,7 +1550,7 @@
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Multi-factor authentication and tested backups do not appear to be consistently in place. Most cyber carriers now treat these as minimum requirements.</t>
+          <t>Tenant, applicant, or investor data appears to be held without a data security program. Cyber carriers treat MFA and encryption as minimum requirements.</t>
         </is>
       </c>
     </row>
@@ -1554,13 +1570,13 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Payment &amp; wire controls</t>
+          <t>Funds transfer security</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>How are changes to vendor bank details and outgoing wire requests verified?</t>
+          <t>How is the flow of funds controlled: rent collection, security deposits, vendor payments, wires, and changes to vendor bank details?</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
@@ -1578,7 +1594,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Vendor bank-detail changes and wires may be released on an email or phone request alone, which is the most common path for social-engineering losses.</t>
+          <t>Wires and vendor bank-detail changes may be released on an email or phone request alone, which is the most common path for social-engineering losses in property operations.</t>
         </is>
       </c>
     </row>
@@ -1598,16 +1614,20 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Safety &amp; training</t>
+          <t>Inspections, life safety &amp; maintenance</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>How are safety programs, training, and inspections documented?</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr"/>
+          <t>How are property inspections, life-safety systems, lighting, and preventive maintenance documented across the portfolio?</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Documented inspections and maintenance logs are what carriers credit; practices that exist only in the property manager's head do not count.</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="n">
         <v>3</v>
       </c>
@@ -1636,13 +1656,13 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Incident reporting</t>
+          <t>Claim intake &amp; reporting</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>What happens when an incident or potential claim occurs?</t>
+          <t>What policies and procedures make sure incidents at the properties (injuries, fires, water losses, tenant claims) are reported and managed properly?</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
@@ -1660,7 +1680,7 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Incidents appear to be reported inconsistently or late. Late reporting is a frequent driver of higher claim costs and coverage disputes.</t>
+          <t>Incidents appear to be reported inconsistently or late. Late reporting is a frequent driver of higher claim costs and coverage disputes, especially on liability claims.</t>
         </is>
       </c>
     </row>
@@ -1680,16 +1700,20 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Open claim review</t>
+          <t>Claims management &amp; advocacy</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>How often are open claims and reserves reviewed with your broker or carrier?</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
+          <t>How are open claims, reserves, carrier-assigned counsel, and public adjusters managed?</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>The workshop asks whether your broker has a systematic process: frequency of updates, claims positioning, policy review, legal guidance, and advocacy.</t>
+        </is>
+      </c>
       <c r="H12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1724,7 +1748,7 @@
       <c r="E13" s="4" t="inlineStr"/>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>After an incident, how are root causes identified and corrective actions tracked?</t>
+          <t>After an incident at a property, how are root causes identified and corrective actions tracked?</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
@@ -1756,21 +1780,21 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Signed contracts</t>
+          <t>Vendor &amp; contractor contracts</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Before work begins with customers, vendors, or subcontractors, how consistently are written contracts in place?</t>
+          <t>Tell us about the contracts you use with vendors and contractors at the properties (snow and ice, landscaping, security, renovations). Are master agreements in place with key vendors?</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr"/>
       <c r="H14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>2</v>
@@ -1794,13 +1818,13 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Insurance requirements</t>
+          <t>Insurance requirements in leases &amp; contracts</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>How do you determine what insurance to require from the parties you work with, and what they require from you?</t>
+          <t>How are insurance requirements set for tenants in leases and for vendors in contracts, and how are lender and management-agreement requirements on you tracked?</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
@@ -1832,13 +1856,13 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Certificate verification</t>
+          <t>Certificate tracking</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>How are certificates of insurance and endorsements (additional insured, waiver of subrogation) verified?</t>
+          <t>What is your process for vetting vendors and contractors who work at the properties, and how are certificates of insurance and endorsements tracked?</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -1846,7 +1870,7 @@
         <v>3</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>2</v>
@@ -1856,7 +1880,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Certificates of insurance are collected but not reviewed, so contractual risk transfer may not be operating when a loss occurs.</t>
+          <t>Vendor certificates of insurance are collected but not reviewed, so the indemnity and additional-insured protection in your contracts may not be operating when a loss occurs.</t>
         </is>
       </c>
     </row>
@@ -1876,18 +1900,18 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Annual risk review</t>
+          <t>Frequent risk assessment</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Does leadership conduct a structured risk review outside of the insurance renewal?</t>
+          <t>How often is a thorough risk assessment of the portfolio performed outside of an insurance policy renewal?</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>A risk review looks at operations, contracts, and controls, not just the policies being renewed.</t>
+          <t>A risk review looks at operations, contracts, properties, and controls, not just the policies being renewed.</t>
         </is>
       </c>
       <c r="H17" s="4" t="n">
@@ -1918,13 +1942,13 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Regulatory monitoring</t>
+          <t>Regulatory &amp; compliance monitoring</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>How are regulatory and compliance changes affecting your operations monitored?</t>
+          <t>How are regulatory and compliance changes affecting the properties monitored (fair housing, ADA, local habitability and safety ordinances, energy and benchmarking rules)?</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -1956,16 +1980,20 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>New activity review</t>
+          <t>New exposure review</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>When you add a new location, product, service, technology, or major customer, is risk and insurance impact reviewed beforehand?</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr"/>
+          <t>When you acquire a property, add a new property type, allow short-term rentals, or add EV charging or lithium-battery storage, is the risk and insurance impact reviewed beforehand?</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>The workshop found owners who had never heard of the lithium-battery exposure and were about to add car chargers.</t>
+        </is>
+      </c>
       <c r="H19" s="4" t="n">
         <v>2</v>
       </c>
@@ -1994,7 +2022,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Property valuation &amp; building updates</t>
+          <t>Carrier recommendations &amp; building updates</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2004,12 +2032,12 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>For the buildings you own, how are replacement values, business-interruption values, flood exposure, building updates (roof, sprinklers, electrical), and carrier loss-control recommendations documented and tracked?</t>
+          <t>What is your procedure for dealing with insurance company recommendations (sprinklers, wiring, boilers, roofs), and how are building updates and flood exposure documented?</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Carriers issue recommendations after inspections. How you respond to them is part of the underwriting story.</t>
+          <t>Carriers issue recommendations after inspections. Owners who track and close them, and show the carrier, negotiate from strength.</t>
         </is>
       </c>
       <c r="H20" s="4" t="n">
@@ -2030,27 +2058,27 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>operational_controls</t>
+          <t>contractual_risk_transfer</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Fleet &amp; driver controls</t>
+          <t>Management agreements</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>hasVehicles</t>
+          <t>usesThirdPartyManager</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>How are drivers screened and vehicles managed (MVRs, telematics, hired and non-owned auto)?</t>
+          <t>How do your management agreements address insurance and indemnification obligations between you and the third-party property manager?</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -2058,7 +2086,7 @@
         <v>3</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J21" s="4" t="n">
         <v>2</v>
@@ -2068,7 +2096,7 @@
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>Motor vehicle records do not appear to be run consistently, which commercial auto underwriters treat as a primary control.</t>
+          <t>Insurance and indemnification terms in the property-management agreement have not been reviewed, so it is unclear who is covered for a loss at a managed property.</t>
         </is>
       </c>
     </row>
@@ -2078,17 +2106,17 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>contractual_risk_transfer</t>
+          <t>operational_controls</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor &amp; vendor risk transfer</t>
+          <t>Snow &amp; ice, security, and site vendors</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -2098,15 +2126,15 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>For subcontractors and vendors, how consistently are indemnity terms, additional-insured status, and waivers of subrogation obtained and enforced?</t>
+          <t>For snow and ice removal, security patrols, and other on-site vendors, how consistently are procedures documented and risk transferred (logs, cameras, indemnity, additional-insured status)?</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
       <c r="H22" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>2</v>
@@ -2120,7 +2148,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2130,25 +2158,25 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Sensitive data handling</t>
+          <t>Leasing, renters insurance &amp; fair housing</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>storesSensitiveData</t>
+          <t>hasResidentialTenants</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>For the sensitive customer, employee, or payment data you hold, how are access, vendor security, and incident response managed?</t>
+          <t>For residential tenants, how are leasing and screening, renters-insurance verification, anti-discrimination training, and short-term-rental monitoring handled?</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
       <c r="H23" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J23" s="4" t="n">
         <v>2</v>
@@ -2182,12 +2210,12 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>With a workforce of this size, how are workers' compensation return-to-work, employment practices (handbook, training, documentation), and benefits data protection handled?</t>
+          <t>With on-site and corporate staff of this size, how are workers' compensation return-to-work, employment practices (handbook, training, documentation), and manager training handled?</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>
       <c r="H24" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I24" s="4" t="n">
         <v>3</v>
@@ -2214,7 +2242,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Board &amp; investor governance</t>
+          <t>Investors, funds &amp; lenders</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2224,12 +2252,12 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>With outside investors or a board, how are directors &amp; officers, fiduciary, and governance-related exposures reviewed?</t>
+          <t>With outside investors, funds, or lenders, how are investor reporting, fund and entity E&amp;O and D&amp;O exposures, and lender insurance requirements managed?</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr"/>
       <c r="H25" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>2</v>
@@ -2246,7 +2274,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2256,22 +2284,22 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Regulated materials &amp; environmental</t>
+          <t>Environmental risks</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>regulatedMaterials</t>
+          <t>environmentalExposures</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>For regulated materials or processes, how are environmental permits, storage practices, and pollution exposure managed?</t>
+          <t>What are your practices for environmental risks at the properties (lead, mold, asbestos, oil tanks, legionella, soil contamination), including due diligence on acquisitions?</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26" s="4" t="n">
         <v>3</v>
@@ -2344,7 +2372,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>About 60 days out, but it varies year to year</t>
+          <t>About 60 days out; we ask brokers to market and follow up 30 days out</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2387,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>90+ days out with a written timeline</t>
+          <t>90+ days out with a written timeline and an updated statement of values</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2402,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>120+ days out with a documented calendar, owners, and a pre-renewal strategy meeting</t>
+          <t>120+ days out with a documented calendar, owners, a pre-renewal strategy meeting, and a reconciled statement of values</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2417,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>No single owner; whoever the broker contacts handles it</t>
+          <t>No single owner; whoever the broker contacts handles it, or the property manager decides</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2447,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>A named owner with defined responsibilities</t>
+          <t>A named owner with defined responsibilities, including certificates and mid-term changes</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2462,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>A named owner, a backup, and a cross-functional review (finance, operations, HR/safety)</t>
+          <t>A named owner, a backup, and a defined split of duties with the property manager, asset management, and finance</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2477,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>We renew the same limits without discussion</t>
+          <t>We trust the agent or go with past numbers; limits follow the premium budget</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2492,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>The broker recommends and we generally accept</t>
+          <t>We have discussed limits with the agent but never worked through examples or lender requirements in detail</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2507,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>We review limits against contracts, assets, and revenue annually</t>
+          <t>We review limits annually against lender and lease requirements, asset values, and revenue</t>
         </is>
       </c>
     </row>
@@ -2494,7 +2522,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>We document the rationale for each limit and deductible and revisit it when the business changes</t>
+          <t>A formal annual process considers industry trends, risk tolerance, balance sheet, defensibility, lender covenants, and documents the rationale for each limit and deductible</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2537,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>We use last year's numbers unless someone flags a change</t>
+          <t>We don't analyze replacement cost; the insurer dictates it and values are carried forward</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2552,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>We update the big items but rarely reconcile schedules</t>
+          <t>We reviewed values a few years ago but do not update often and are not confident in the process</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2567,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Finance validates values annually against records</t>
+          <t>Values and building details are updated annually and checked against recent construction costs</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2582,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Values are reconciled against financials, fixed-asset registers, and schedules, with sign-off before submission</t>
+          <t>Values are updated annually, reconciled against rebuilds, appraisals, and recent claims, with construction, protection, and update history documented per building</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2612,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>We mention major changes when we remember</t>
+          <t>We mention major acquisitions or sales when we remember</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2627,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>A defined process captures changes and shares them with the broker</t>
+          <t>A defined process reports each acquisition, disposition, and major renovation to the broker with values and lender requirements</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2642,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Changes are logged, reviewed quarterly for insurance impact, and reflected in mid-term endorsements when needed</t>
+          <t>Changes are logged, reviewed quarterly for insurance impact, and reflected in schedules and endorsements when they happen</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2657,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>None; we sign applications and the broker handles the rest</t>
+          <t>I don't know; we have never seen what brokers present to market</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2672,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>We submit updated information annually but have not seen how our story is told to carriers</t>
+          <t>We submit updated information annually and confirm the broker understands changes to the portfolio</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2687,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>We review the submission and know which carriers quoted or declined</t>
+          <t>We review the submission and know which carriers quoted or declined and why</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2702,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>We collaborate with our broker on how best to portray the company in the marketplace, review the full submission, and receive a market summary with reasons for declinations</t>
+          <t>We collaborate with our broker to determine how best to portray the portfolio, review the full submission and narrative, and receive a market summary with reasons for declinations</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2717,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Basic antivirus; MFA and tested backups are not consistently in place</t>
+          <t>No data security program or process; information is stored locally and not encrypted</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2732,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>MFA on email; backups exist but are not tested regularly</t>
+          <t>Some form of data security, such as limited access, encryption, or occasional employee education</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2747,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>MFA on email and remote access, tested offline backups, endpoint detection, and a written incident plan</t>
+          <t>A formal data security program: MFA, encryption, limited access, regular training, and a written incident plan</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2762,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>All of the prior plus annual testing, vendor security review, and executive reporting</t>
+          <t>Formal program plus vendor security review of property-management and payment platforms, tested backups, and annual review with the broker</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2777,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>No formal protocol; an email or phone request is usually sufficient</t>
+          <t>No formal protocols; an email or phone request is usually sufficient</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2807,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Written procedure with callback verification to a known number and dual approval for all bank changes and wires</t>
+          <t>Written procedures with callback verification to a known number and dual approval for wires and bank-detail changes</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2822,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Formal written program with regular training: dual authorization, callback verification, destination confirmation, and receipt confirmation</t>
+          <t>Formal written program with regular training: dual authorization, calls to verify, destination-detail confirmation, receipt confirmation, and periodic consultation with the bank on best practices</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2837,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Training happens on the job; little is written down</t>
+          <t>Inspections happen when something breaks; little is written down</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2852,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Some written procedures; training records are incomplete</t>
+          <t>Some written procedures; inspection and maintenance records are incomplete or live only with the manager</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2867,7 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Written safety program, documented training, and periodic inspections</t>
+          <t>Written inspection schedule, life-safety testing records, and a preventive maintenance plan per property</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2882,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Written program with documented training, inspections, near-miss reporting, and management review of results</t>
+          <t>Written program with documented inspections, life-safety testing, lighting and security logs, preventive maintenance plans, and ownership review of results</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2897,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>It is reported when someone thinks of it, sometimes weeks later</t>
+          <t>No policies or protocols; the property manager reports claims directly to the carrier when they think of it</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2912,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Supervisors know to report, but timing and format vary</t>
+          <t>Supervisors and managers know to report, but timing and format vary; we check in with the broker when we need an update</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2927,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>A written protocol defines who reports, how, and within what timeframe</t>
+          <t>A written protocol defines who reports, how, and within what timeframe, with an incident form for every event</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2942,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Written protocol, reporting within 24–48 hours, an incident form, and tracking of every report</t>
+          <t>Written protocol, reporting within 24–48 hours, incident forms, and formal meetings with broker and adjusters on a predetermined timeline</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2957,7 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>We do not review open claims</t>
+          <t>We work directly with the carrier and adjuster; we do not focus on the liability claims process or communicate with assigned counsel</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2972,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Only when the carrier or broker raises something</t>
+          <t>We engage the broker if we are not satisfied; the broker primarily deals with counsel while we monitor open claims</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2987,7 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Scheduled reviews at least twice a year</t>
+          <t>Scheduled claim reviews at least twice a year with reserve discussion; we consider a public adjuster case by case</t>
         </is>
       </c>
     </row>
@@ -2974,7 +3002,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Quarterly claim reviews with reserve challenges, adjuster accountability, and pre-renewal loss-run reconciliation</t>
+          <t>A systematic process: quarterly reviews with reserve challenges, pre-assigned preferred defense counsel where possible, public-adjuster decisions made with the broker against policy wording, and pre-renewal loss-run reconciliation</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3032,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Supervisors discuss causes; actions are not tracked</t>
+          <t>The property manager discusses causes; actions are not tracked</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3047,7 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Root-cause review for significant incidents with documented corrective actions</t>
+          <t>Root-cause review for significant incidents with documented corrective actions and work orders</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3062,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Every incident gets a root-cause review, corrective actions are tracked to closure, and trends are reported to leadership</t>
+          <t>Every incident gets a root-cause review, corrective actions are tracked to closure across the portfolio, and trends are reported to ownership</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3077,7 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Often work starts on a handshake or PO alone</t>
+          <t>We don't always get contracts signed; work often starts on a proposal or a call</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3092,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Contracts exist for major relationships; smaller ones vary</t>
+          <t>An attorney reviews or writes contracts and we make sure they are signed</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3107,7 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Signed contracts are required before work begins</t>
+          <t>Attorney-reviewed contracts plus broker review for insurance and risk-transfer terms; signed before work starts</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3122,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Signed contracts required, with standard indemnity and insurance language reviewed by counsel and tracked centrally</t>
+          <t>Attorney and broker review, signed before work starts, master agreements with key vendors, and payment blocked when contract or insurance terms are missing</t>
         </is>
       </c>
     </row>
@@ -3109,7 +3137,7 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>We do not set requirements; we accept whatever the other party proposes</t>
+          <t>We do not set requirements; we accept whatever the tenant, vendor, or lender proposes</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3152,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>We use a generic requirement list without reviewing it</t>
+          <t>We use generic lease and contract language without reviewing it</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3167,7 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Requirements are defined by relationship type and reviewed by broker or counsel</t>
+          <t>Requirements are defined by relationship type (tenant, vendor, contractor) and reviewed by broker or counsel</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3182,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Requirements are defined, reviewed annually, and cross-checked against our own policies and customer demands</t>
+          <t>Requirements are defined, reviewed annually, cross-checked against our own policies and every lender and management-agreement obligation, and enforced</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3197,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>We collect certificates when asked but do not review them</t>
+          <t>We don't; certificates are collected when asked and not reviewed</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3212,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Someone checks that a certificate exists; endorsements are rarely verified</t>
+          <t>We obtain certificates with additional-insured status and check coverage and limit adequacy, but tracking is manual and infrequent</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3227,7 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Certificates and required endorsements are verified before work and on expiration</t>
+          <t>Certificates and required endorsements are verified before work and on expiration, in a tracking system</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3242,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Verification is tracked in a system, endorsements are matched to contract terms, and non-compliance is escalated</t>
+          <t>Software tracks every vendor's insurance in real time, the broker reviews complete policies for key contractors, endorsements are matched to contract terms, and non-compliant vendors are stopped from working</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3272,7 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>More than 18 months ago, or only when a new broker or agent first came on board</t>
+          <t>More than 18 months ago, or only when a new agent first came on board</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3287,7 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>An annual risk review with a documented risk list</t>
+          <t>Annually, with a documented list of risks by property</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3302,7 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Annual review with owners, action plans, and quarterly progress updates to leadership</t>
+          <t>Annually with owners and action plans, reviewed with the broker so prevention, mitigation, and insurance stay aligned</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3317,7 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>We learn about changes when we are notified of a violation or audit</t>
+          <t>We learn about changes when we are notified of a violation, complaint, or audit</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3347,7 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>A defined owner monitors regulations and briefs leadership</t>
+          <t>A defined owner monitors regulations, and required training and postings are documented</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3362,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Defined owner, documented compliance calendar, and periodic compliance audits</t>
+          <t>Defined owner, documented compliance calendar, annual training with records, and periodic compliance audits with counsel</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3392,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Sometimes, for very large changes</t>
+          <t>Sometimes, for very large acquisitions</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3407,7 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>A review step is included in the launch process</t>
+          <t>A review step with the broker is part of acquisition due diligence and major operational changes</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3422,7 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Documented pre-launch review with operations, finance, broker input, and follow-up after launch</t>
+          <t>Documented pre-acquisition and pre-launch review (environmental due diligence, valuation, lender requirements, new exposures) with follow-up after closing</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3437,7 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Values are carried forward; building updates and carrier recommendations are not tracked</t>
+          <t>We do as little as possible; updates and flood zones are not documented</t>
         </is>
       </c>
     </row>
@@ -3424,7 +3452,7 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Values were reviewed a few years ago; we do the minimum needed to stay compliant with carrier recommendations</t>
+          <t>We do the bare minimum to stay compliant with the insurer; updates are partially documented</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3467,7 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Replacement and BI values are reviewed annually; update history and recommendation responses are documented</t>
+          <t>An active protocol responds to and tracks recommendations; roof, sprinkler, electrical, and boiler updates are documented with dates</t>
         </is>
       </c>
     </row>
@@ -3454,14 +3482,14 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Professional valuation within three years, BI worksheet, flood zone determination, documented inspections and update history, and an active protocol for responding to and tracking every carrier recommendation</t>
+          <t>Active protocol for every recommendation with completion shown to the carrier, documented update history per building, flood zone determinations, and a professional valuation within three years</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="B78" s="4" t="n">
@@ -3469,14 +3497,14 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>We do not run MVRs consistently; personal vehicle use is not addressed</t>
+          <t>We do not review these requirements in agreements with our property managers</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="B79" s="4" t="n">
@@ -3484,14 +3512,14 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>MVRs at hire only; no written fleet policy</t>
+          <t>We accept the terms and conditions in the manager's boilerplate agreement</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="B80" s="4" t="n">
@@ -3499,14 +3527,14 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Written fleet policy, annual MVRs, and a defined hired/non-owned auto approach</t>
+          <t>Counsel reviewed the agreement; we know who insures what and hold the manager's certificate</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="B81" s="4" t="n">
@@ -3514,14 +3542,14 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Written policy, annual MVRs with disqualification criteria, telematics or cameras, and driver training records</t>
+          <t>We actively review and dictate the insurance and indemnity terms, require adequate limits and coverages from the manager, and regularly request updated certificates to confirm they are in place</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="B82" s="4" t="n">
@@ -3529,14 +3557,14 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>We rely on the vendor's own paperwork</t>
+          <t>Employees or vendors handle it informally; no logs and contracts have not been reviewed</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="B83" s="4" t="n">
@@ -3544,14 +3572,14 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Our agreement includes the terms, but we rarely confirm the endorsements</t>
+          <t>Employees are trained or contractors are hired, but snow logs, security procedures, and contract terms are inconsistent</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="B84" s="4" t="n">
@@ -3559,14 +3587,14 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Terms are standard and endorsements are confirmed before work</t>
+          <t>Every snow removal and patrol is documented, and vendors indemnify and name us as additional insured</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="B85" s="4" t="n">
@@ -3574,14 +3602,14 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Terms are standard, endorsements confirmed, non-compliant vendors are stopped from working, and exceptions are approved in writing</t>
+          <t>Documented logs visible on cameras, written security and snow procedures, contracts reviewed for indemnity and additional-insured terms, and vendor insurance tracked in a compliance system</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="B86" s="4" t="n">
@@ -3589,14 +3617,14 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Access is broad; we have not reviewed vendor security or an incident plan</t>
+          <t>No formal process; renters insurance is not tracked and fair-housing training is informal</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="B87" s="4" t="n">
@@ -3604,14 +3632,14 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Access is limited informally; incident response is undocumented</t>
+          <t>Application with employment verification and some screening; renters insurance tracked manually and updated infrequently; handbook statement only</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="B88" s="4" t="n">
@@ -3619,14 +3647,14 @@
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Role-based access, vendor security review, and a written incident response plan</t>
+          <t>Attorney-vetted application and lease, background checks, renters insurance required and tracked, annual fair-housing training, lease prohibits short-term rentals</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="B89" s="4" t="n">
@@ -3634,7 +3662,7 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>All of the prior plus annual tabletop exercises, data inventory, and breach-notification readiness</t>
+          <t>All of the prior plus software that monitors renters insurance in real time and force-places when missing, documented annual training with counsel consultation, and active monitoring for short-term rental use</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3722,7 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>All of the prior plus experience-mod review, claims-trend analysis, and annual employment-practices training</t>
+          <t>All of the prior plus experience-mod review, claims-trend analysis, and annual employment-practices training with records</t>
         </is>
       </c>
     </row>
@@ -3709,7 +3737,7 @@
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>They have not been reviewed</t>
+          <t>Updates are provided on demand; entity coverages and lender requirements have not been reviewed</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3752,7 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Coverage was placed at the time of investment and not revisited</t>
+          <t>Annual performance updates; coverage was placed at the time of the raise and not revisited</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3767,7 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Reviewed annually with the broker against bylaws, investor agreements, and benefit plans</t>
+          <t>Quarterly reporting on performance and key metrics; E&amp;O and D&amp;O reviewed annually with the broker against fund documents; lender requirements tracked</t>
         </is>
       </c>
     </row>
@@ -3754,14 +3782,14 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Annual review plus board reporting on limits, indemnification agreements, and fiduciary controls</t>
+          <t>Quarterly reporting with online access, annual review of entity coverages, every legal entity confirmed as a named insured, and lender requirements reconciled at each closing</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="B98" s="4" t="n">
@@ -3769,14 +3797,14 @@
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>We are not sure what permits apply; storage practices are informal</t>
+          <t>I don't know; we have not looked at it</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="B99" s="4" t="n">
@@ -3784,14 +3812,14 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Permits are in place; documentation of storage and disposal is inconsistent</t>
+          <t>We depend on what we read and hear from industry groups; we may purchase environmental insurance</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="B100" s="4" t="n">
@@ -3799,14 +3827,14 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Permits, storage, and disposal are documented with a compliance owner</t>
+          <t>An environmental specialist has reviewed the portfolio and surveys; environmental due diligence is part of acquisitions</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="B101" s="4" t="n">
@@ -3814,7 +3842,7 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Documented compliance program, periodic environmental audits, and pollution exposure reviewed with the broker</t>
+          <t>Specialist reviews the portfolio routinely, moisture and mold procedures are written, lender environmental conditions are tracked, and environmental insurance is reviewed with the broker</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3868,31 +3896,35 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr"/>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>For a 3PL this includes the value of customers' goods in your care, custody, and control, vehicle and trailer schedules, and square footage by location.</t>
+          <t>Include unit counts, rent roll and business-income values, and any building improvements since the last valuation.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>mkt_exposure_data</t>
+          <t>ops_safety_training</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr"/>
+          <t>multifamily</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>How are unit and common-area inspections, life-safety systems (smoke and CO detectors, sprinklers, egress), lighting, and preventive maintenance documented across the communities?</t>
+        </is>
+      </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>For a manufacturer this includes machinery and equipment values, a business-interruption worksheet, and any dependence on a single supplier or customer.</t>
+          <t>Habitability claims turn on documentation: inspection logs, work-order completion, and life-safety testing records.</t>
         </is>
       </c>
     </row>
@@ -3904,157 +3936,73 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>How are warehouse and dock safety (forklift certification, racking, housekeeping), fire protection (sprinkler inspections, impairment procedures, commodity storage), and driver training documented?</t>
+          <t>How are roof, sprinkler, electrical, and boiler inspections, life-safety systems, and preventive maintenance documented across the buildings?</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Warehouse underwriters look first at fire protection and forklift and dock injury controls.</t>
+          <t>Roof age, sprinkler impairments, aluminum wiring, and boiler condition are the recommendations carriers issue most often.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>ops_safety_training</t>
+          <t>crt_insurance_requirements</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>How are machine guarding, lockout/tagout, hearing and respiratory protection, and safety training documented?</t>
-        </is>
-      </c>
+          <t>cre_owner</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Machine guarding and lockout/tagout drive both workers' compensation experience and product-safety credibility with underwriters.</t>
+          <t>Commercial leases typically require tenant liability and property coverage with the owner as additional insured; lenders require specific limits, mortgagee clauses, and flood where applicable.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>crt_signed_contracts</t>
+          <t>crt_insurance_requirements</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Before goods are received or work begins, how consistently are written warehousing agreements, customer contracts, and carrier/vendor agreements in place?</t>
-        </is>
-      </c>
+          <t>multifamily</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Warehouse receipts and customer contracts define your legal liability for goods in your care. Unsigned or inconsistent terms are a common gap.</t>
+          <t>Vendor requirements matter most here: snow and ice, security, and renovation contractors should indemnify and name the owner and manager as additional insureds.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>crt_signed_contracts</t>
+          <t>emr_regulatory</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>How consistently are written supply agreements, customer purchase terms, and vendor contracts in place before production or shipment begins?</t>
-        </is>
-      </c>
+          <t>multifamily</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Customer terms often carry product warranty, recall, and indemnity obligations that shape your liability program.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>crt_insurance_requirements</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>logistics_3pl</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Customers commonly require warehouse legal liability, cargo, and auto limits. Carriers and subcontracted haulers should be held to defined requirements in return.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>crt_insurance_requirements</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Large customers often specify product liability limits and vendor endorsements; suppliers should be held to defined requirements for the components they provide.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>emr_new_activity_review</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>logistics_3pl</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>When you take on a new commodity, temperature-controlled or hazardous storage, a new customer contract, or a new facility, is risk and insurance impact reviewed beforehand?</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>emr_new_activity_review</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>When you launch a new product, add a production line or process, or enter a new market, is product liability, recall, and business-interruption impact reviewed beforehand?</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr"/>
+          <t>Fair-housing training records, required postings, and consistent screening criteria are the first things asked about in a discrimination claim.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4067,7 +4015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4132,17 +4080,17 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Your renewal process may begin too late to fully document your risk controls.</t>
+          <t>Your renewal process may begin too late to fully document the portfolio.</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Renewal preparation appears to begin with limited runway. Controls that are not documented in time rarely make it into the submission carriers evaluate.</t>
+          <t>Renewal preparation appears to begin with limited runway. Updated values, building improvements, and closed carrier recommendations that are not documented in time rarely make it into the submission carriers evaluate.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Benchmark indication: high-impact underwriting strengths were identified elsewhere in your answers, but they may not be incorporated consistently into carrier submissions.</t>
+          <t>Benchmark indication: strengths were identified elsewhere in your answers, but they may not be incorporated consistently into what carriers see.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -4167,17 +4115,17 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Your contracts and insurance-verification process may not be operating as one control system.</t>
+          <t>Your leases, vendor contracts, and certificate tracking may not be operating as one control system.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Answers about signed contracts, insurance requirements, and certificate verification are uneven. Risk transfer only works when all three align.</t>
+          <t>Answers about signed vendor contracts, insurance requirements, and certificate verification are uneven. Risk transfer only works when the requirement, the contract, and the certificate line up.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: review whether contractual requirements, certificates of insurance, and policy endorsements align for your largest customer and vendor relationships.</t>
+          <t>Potential opportunity: review whether lease and contract requirements, certificates of insurance, and endorsements align for your largest tenants and your snow, security, and renovation vendors.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -4202,17 +4150,17 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Your business has changed faster than your insurance-governance process.</t>
+          <t>Your portfolio has changed faster than your insurance-governance process.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>You reported recent acquisitions or new locations, but operational changes reach the insurance program late or inconsistently.</t>
+          <t>You reported recent acquisitions, dispositions, or major renovations, but portfolio changes reach the insurance program late or inconsistently.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Areas to investigate: new locations, increased payroll, new services, and updated property values, and whether each is reflected in current schedules.</t>
+          <t>Areas to investigate: newly acquired properties, updated replacement values, lender requirements at each closing, and whether renovations are reflected in schedules.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -4242,12 +4190,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Incident reporting, open-claim review, or corrective-action tracking appear informal. Claims that are not managed tend to cost more and stay open longer.</t>
+          <t>Incident reporting, open-claim review, or corrective-action tracking appear informal, and there is no systematic broker process for advocacy, counsel, or public adjusters.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: evaluate reporting timelines, reserve review, adjuster accountability, and how corrective actions are tracked to closure.</t>
+          <t>Potential opportunity: evaluate reporting timelines, reserve review, carrier-assigned counsel, public-adjuster decisions, and how corrective actions are tracked across properties.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -4272,17 +4220,17 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Incomplete exposure data or a weak underwriting narrative could limit your market options.</t>
+          <t>A statement of values that carriers do not trust, or a story they never hear, could limit your market options.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Exposure values appear to be carried forward without reconciliation, or you have limited visibility into what carriers receive.</t>
+          <t>Replacement costs appear to be dictated by the insurer or carried forward, or you have limited visibility into what carriers receive about the portfolio.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Pricing cannot be assessed from this questionnaire alone. However, carriers generally offer their best terms to accounts that present validated data and a clear narrative, subject to policy, loss, and underwriting review.</t>
+          <t>Pricing cannot be assessed from this questionnaire alone. However, carriers generally offer their best terms to portfolios that present validated values, documented building updates, and a clear narrative, subject to policy, loss, and underwriting review.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -4307,17 +4255,17 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Payment-change and wire controls may leave a path open for social-engineering losses.</t>
+          <t>Funds-transfer controls may leave a path open for social-engineering losses.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Vendor bank-detail changes or wires may be released without callback verification and dual approval. This is the most common route for funds-transfer fraud.</t>
+          <t>Wires, vendor bank-detail changes, or security-deposit returns may be released without callback verification and dual approval. This is the most common route for funds-transfer fraud in property operations.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: confirm callback procedures, approval thresholds, and whether crime or cyber coverage includes social-engineering terms, subject to policy review.</t>
+          <t>Potential opportunity: confirm callback procedures, approval thresholds, controls at the property-management company, and whether crime or cyber coverage includes social-engineering terms, subject to policy review.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -4342,22 +4290,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Cyber controls may not meet the minimums that most carriers now require.</t>
+          <t>Protection of tenant, applicant, and investor data may not meet the minimums cyber carriers now require.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Multi-factor authentication, tested backups, and a written incident plan are the controls cyber underwriters ask about first.</t>
+          <t>Multi-factor authentication, encryption, tested backups, and a written incident plan are the controls cyber underwriters ask about first, along with the security of your property-management platform.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: document current controls, close gaps before the next cyber application, and confirm which controls are attested on existing applications.</t>
+          <t>Potential opportunity: document current controls, review the property-management and payment vendors' security, and confirm which controls are attested on existing applications.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>ops_cyber_controls, br_data_security</t>
+          <t>ops_cyber_controls</t>
         </is>
       </c>
     </row>
@@ -4377,17 +4325,17 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Insurance program ownership appears informal.</t>
+          <t>Insurance program ownership appears informal or split with the property manager.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Without a named owner and defined responsibilities, renewal tasks, certificate requests, and mid-term changes tend to fall through the cracks.</t>
+          <t>Without a named owner and a defined split of duties, certificate requests, mid-term acquisitions, and lender requirements tend to fall through the cracks.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: assign an owner and backup, and define the touchpoints with finance, operations, and HR/safety.</t>
+          <t>Potential opportunity: assign an owner and backup, and define who handles certificates, closings, and claims between ownership and the manager.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -4412,17 +4360,17 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Limits and deductibles appear to be renewed without a documented rationale.</t>
+          <t>Limits and deductibles appear to follow the budget rather than a documented rationale.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>This diagnostic does not assess whether limits are adequate. It does note that limits which are never revisited may not track contract requirements or asset growth.</t>
+          <t>This diagnostic does not assess whether limits are adequate. It does note that limits which are never revisited may not track lender covenants, lease requirements, or portfolio growth.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: document the basis for each limit and deductible with a licensed advisor and revisit it when contracts or assets change.</t>
+          <t>Potential opportunity: document the basis for each limit and deductible with a licensed advisor, including key liability cases and lender requirements, and revisit it as the portfolio changes.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -4447,17 +4395,17 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Safety and training practices may exist but are not documented in a form underwriters can credit.</t>
+          <t>Inspection, life-safety, and maintenance practices may exist but are not documented in a form underwriters can credit.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Written programs, training records, and inspection logs are what carriers use to distinguish a well-run operation from an average one.</t>
+          <t>Inspection schedules, life-safety testing records, lighting logs, and preventive maintenance plans are what carriers use to distinguish a well-run portfolio from an average one.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: assemble a safety documentation package before the next submission.</t>
+          <t>Potential opportunity: assemble an inspection and maintenance documentation package per property before the next submission.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -4478,21 +4426,21 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Owned-property values and building updates may be undocumented.</t>
+          <t>Carrier recommendations and building updates may not be tracked or shown to the market.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Replacement cost, business-interruption values, flood exposure, and building-system updates drive both coverage terms and pricing conversations.</t>
+          <t>How you respond to sprinkler, wiring, boiler, and roof recommendations, and whether updates and flood exposure are documented, drives both coverage terms and pricing conversations.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Areas to investigate: date of last valuation, BI worksheet, flood zone determination, and documented roof, sprinkler, and electrical updates.</t>
+          <t>Areas to investigate: open recommendations by property, completion evidence, roof and system update dates, flood zone determinations, and the date of the last professional valuation.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -4504,47 +4452,47 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>fleet_controls</t>
+          <t>management_agreement_gap</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>operational_controls</t>
+          <t>contractual_risk_transfer</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Fleet and driver controls may not be documented to the level auto underwriters expect.</t>
+          <t>The insurance and indemnity terms in your property-management agreement may not have been reviewed.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>MVR practices, fleet policy, and hired/non-owned auto handling are primary controls for commercial auto.</t>
+          <t>Boilerplate management agreements often leave it unclear who insures what and who indemnifies whom when a loss occurs at a managed property.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: adopt a written fleet policy with annual MVRs and disqualification criteria.</t>
+          <t>Potential opportunity: have counsel and the broker review the agreement, dictate required limits and coverages, and hold current certificates from the manager.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>subcontractor_transfer_gap</t>
+          <t>site_vendor_gap</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>contractual_risk_transfer</t>
+          <t>operational_controls</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -4552,29 +4500,29 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor and vendor risk transfer may not be enforced.</t>
+          <t>Snow and ice, security, and site-vendor procedures may not be documented or transferring risk.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Indemnity terms and endorsements that are not confirmed before work begins may not respond when a loss occurs.</t>
+          <t>Slip-and-fall and premises claims turn on logs, cameras, and whether the vendor's contract indemnifies and insures you.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: confirm additional-insured and waiver endorsements for active vendors.</t>
+          <t>Potential opportunity: require documented snow logs and patrol procedures, and confirm indemnity and additional-insured terms for every site vendor.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>workforce_programs_gap</t>
+          <t>residential_programs_gap</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -4583,129 +4531,164 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Workforce programs (return-to-work, handbook, manager training) may be informal for a company of your size.</t>
+          <t>Leasing, renters-insurance, and fair-housing practices may be informal for the size of the residential portfolio.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>These programs influence workers' compensation experience and employment-practices exposure.</t>
+          <t>Renters insurance that is not tracked, screening that is not consistent, and training that is not documented all show up in liability and discrimination claims.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: document return-to-work procedures and update the employee handbook.</t>
+          <t>Potential opportunity: evaluate real-time renters-insurance monitoring, attorney-vetted lease and screening criteria, and documented annual fair-housing training.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>br_workforce_programs</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>investor_governance_gap</t>
+          <t>workforce_programs_gap</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>operational_controls</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Board and investor-related exposures may not have been reviewed since the investment.</t>
+          <t>Workforce programs (return-to-work, handbook, manager training) may be informal for a staff of your size.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Directors &amp; officers, fiduciary, and indemnification arrangements are typically revisited as ownership and boards change.</t>
+          <t>These programs influence workers' compensation experience and employment-practices exposure across on-site teams.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: review governance-related exposures with a licensed advisor against current bylaws and investor agreements.</t>
+          <t>Potential opportunity: document return-to-work procedures and update the employee handbook.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>br_governance_investors</t>
+          <t>br_workforce_programs</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>environmental_gap</t>
+          <t>investor_governance_gap</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>emerging_risk</t>
+          <t>governance</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Environmental compliance and pollution exposure may not be documented.</t>
+          <t>Investor, fund, and lender-related exposures may not have been reviewed since the last capital event.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Permits, storage practices, and disposal records are the starting point for any environmental conversation with carriers.</t>
+          <t>Fund and entity E&amp;O and D&amp;O, named-insured completeness across every LLC, and lender requirements are typically revisited as deals close and boards change.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Areas to investigate: applicable permits, storage documentation, and whether pollution exposure has been reviewed.</t>
+          <t>Potential opportunity: review entity coverages with a licensed advisor against fund documents and confirm every legal entity is scheduled as a named insured.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_governance_investors</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>environmental_gap</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>emerging_risk</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Environmental exposures at the properties may not have been reviewed.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Lead, mold, asbestos, oil tanks, legionella, and soil conditions are the starting point for any environmental conversation with carriers and lenders.</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Areas to investigate: environmental surveys on file, acquisition due diligence, moisture and mold procedures, lender environmental conditions, and whether pollution exposure has been reviewed.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>br_environmental</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>emerging_risk_unmanaged</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>emerging_risk</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C19" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>New activities and regulatory changes may reach the insurance program after the fact.</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Without a pre-launch review step, new locations, products, and technology can create exposures that are not reflected until the next renewal.</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Potential opportunity: add a risk and insurance checkpoint to your launch process.</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Acquisitions, regulatory changes, and new exposures may reach the insurance program after the fact.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Without a pre-acquisition and pre-launch review step, new properties, short-term rentals, EV charging, and lithium-battery storage can create exposures that are not reflected until the next renewal.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Potential opportunity: add a risk and insurance checkpoint to acquisition due diligence and to operational changes at the properties.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>emr_new_activity_review, emr_regulatory, emr_annual_review</t>
         </is>
@@ -4790,7 +4773,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>How ready is your company to be evaluated by the insurance market?</t>
+          <t>How ready is your real estate portfolio to be evaluated by the insurance market?</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -4800,7 +4783,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>CFOs, COOs, and owners unsure whether the company is presenting an accurate, differentiated risk story.</t>
+          <t>Owners, asset managers, and CFOs unsure whether the portfolio is presenting an accurate, differentiated risk story.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr"/>
@@ -4820,17 +4803,17 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Is your next renewal on a timeline, or on autopilot?</t>
+          <t>Is your property renewal on a timeline, or on autopilot?</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>A confidential check of your renewal runway, the data carriers will ask for, and the changes that need to be documented before submissions go out.</t>
+          <t>A confidential check of your renewal runway, the statement of values carriers will scrutinize, and the acquisitions and updates that need to be documented before submissions go out.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>CFOs and risk managers facing a renewal within three to nine months.</t>
+          <t>Owners, asset managers, and CFOs facing a property renewal within three to nine months.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -4845,7 +4828,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Timing, data, and the story carriers receive. These answers determine whether preparation starts early enough to matter.</t>
+          <t>Timing, values, and the story carriers receive. These answers determine whether preparation starts early enough to matter.</t>
         </is>
       </c>
     </row>
@@ -4862,17 +4845,17 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Are your contracts actually transferring risk, or just describing it?</t>
+          <t>Are your leases and vendor contracts actually transferring risk, or just describing it?</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>A confidential scan of how signed contracts, insurance requirements, certificates, and subcontractor terms work together as one control system.</t>
+          <t>A confidential scan of how leases, vendor and snow-removal contracts, management agreements, insurance requirements, and certificate tracking work together as one control system.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>COOs and CFOs in construction, manufacturing, real estate, and logistics who rely on vendors and subcontractors.</t>
+          <t>Owners and property managers who rely on tenants' insurance and on-site vendors.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -4882,12 +4865,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Your contract-risk workflow</t>
+          <t>Your lease and vendor risk-transfer workflow</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Requirements that are never verified, and certificates that are never matched to contracts, do not transfer risk when a loss occurs.</t>
+          <t>Requirements that are never verified, and certificates that are never matched to leases and contracts, do not transfer risk when a loss occurs.</t>
         </is>
       </c>
     </row>
@@ -4904,17 +4887,17 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Are claims being managed, or just reported?</t>
+          <t>Are claims at your properties being managed, or just reported?</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>A confidential look at reporting speed, open-claim cadence, return-to-work practices, and how corrective actions are tracked.</t>
+          <t>A confidential look at reporting speed, open-claim cadence, public-adjuster and counsel practices, and how corrective actions are tracked across the portfolio.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>CFO, HR, and operations leaders frustrated by recurring or poorly managed claims.</t>
+          <t>Owners, asset managers, and property managers frustrated by recurring or poorly managed claims.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -4929,7 +4912,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Late reporting, unreviewed reserves, and untracked corrective actions are the most common reasons claims cost more and stay open longer.</t>
+          <t>Late reporting, unreviewed reserves, unmanaged counsel, and untracked corrective actions are the most common reasons property claims cost more and stay open longer.</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4990,27 +4973,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>3PL / warehousing / distribution</t>
+          <t>Multifamily / apartment communities</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Fleet, property, cargo, labor, contracts</t>
+          <t>Tenant, premises, discrimination</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Cargo, auto, warehouse legal liability, fire protection</t>
+          <t>Renters insurance, habitability, EPLI, vendor controls</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -5022,59 +5005,59 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>food_cold_storage</t>
+          <t>office</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Food distribution / cold storage</t>
+          <t>Office</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Spoilage and temperature dependency</t>
+          <t>Property values and tenant improvements</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Refrigeration breakdown, recall, contamination</t>
+          <t>SOV quality, lease requirements, BI, life safety</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>industrial_flex</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Light / advanced manufacturing</t>
+          <t>Industrial / flex / warehouse</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Property, machinery, products, WC</t>
+          <t>Large replacement values and tenant operations</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Business interruption, machine guarding, product liability</t>
+          <t>SOV quality, sprinkler and roof condition, tenant contracts, environmental</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -5086,76 +5069,76 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>life_sciences</t>
+          <t>retail_mixed_use</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Life-sciences supplier</t>
+          <t>Retail / mixed-use</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>High-value inventory and regulated work</t>
+          <t>Premises liability and vendor dependence</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Clinical/product liability, cold chain, cyber, E&amp;O</t>
+          <t>Snow and ice, security, lease requirements, liquor tenants</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>contractors</t>
+          <t>net_lease</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Contractor / trades</t>
+          <t>Net-lease / single-tenant</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Subcontracting and contractual risk</t>
+          <t>Lease-driven insurance obligations</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Wrap-ups, fleet, jobsite safety, certificates</t>
+          <t>Tenant compliance tracking, lender requirements, named insureds</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>cre_owners</t>
+          <t>self_storage</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Commercial real estate owner</t>
+          <t>Self-storage</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -5165,12 +5148,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Property values and vendor dependence</t>
+          <t>Property, customer goods, access control</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>SOV quality, flood, BI, leases, management agreements</t>
+          <t>Customer goods legal liability, security, tenant insurance programs</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -5182,12 +5165,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>multifamily</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Multifamily / property manager</t>
+          <t>Hospitality / hotel assets</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -5197,12 +5180,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Tenant, premises, discrimination</t>
+          <t>Property, liquor, events, seasonal labor</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Renters insurance, habitability, EPLI, vendor controls</t>
+          <t>Liquor, pools, events, management agreements, D&amp;O</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -5214,12 +5197,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>healthcare</t>
+          <t>senior_housing</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Healthcare practice / MSO</t>
+          <t>Senior housing / assisted living</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -5229,12 +5212,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Professional, privacy, employment</t>
+          <t>Severe liability and workforce exposure</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Medical professional, cyber, regulatory, credentialing</t>
+          <t>Abuse controls, professional liability, staffing, auto</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -5246,44 +5229,44 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>senior_living</t>
+          <t>student_housing</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Senior living / home care</t>
+          <t>Student housing</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Severe liability and workforce exposure</t>
+          <t>Turnover, premises, parental guarantees</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Abuse controls, auto, professional liability, staffing</t>
+          <t>Renters insurance, security, event and alcohol exposure</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>professional_services</t>
+          <t>association</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Professional services</t>
+          <t>Condo / HOA association</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -5293,12 +5276,12 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>E&amp;O, cyber, executive risk</t>
+          <t>Governance, common areas, D&amp;O</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Contract scope, client concentration, privacy</t>
+          <t>D&amp;O, master policy allocation, vendor controls, reserves</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -5310,76 +5293,76 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>technology_msp</t>
+          <t>third_party_manager</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Technology / MSP</t>
+          <t>Third-party property manager</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Contractual and cyber aggregation</t>
+          <t>Management-agreement exposure across many owners</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Tech E&amp;O, ransomware, dependent business interruption</t>
+          <t>Management agreements, E&amp;O, tenant discrimination, funds handling</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>auto_dealers</t>
+          <t>developer</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Auto dealer / fleet business</t>
+          <t>Developer / owner-builder</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Inventory, garage, drivers</t>
+          <t>Construction and lease-up risk</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Garage liability, false pretense, cyber, weather</t>
+          <t>Builders risk, wrap-ups, contractor certificates, lender requirements</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>hospitality_clubs</t>
+          <t>land</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Hospitality / country club</t>
+          <t>Land / agricultural holdings</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -5389,12 +5372,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Property, liquor, events, seasonal labor</t>
+          <t>Premises and environmental</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Liquor, golf carts, pools, events, D&amp;O</t>
+          <t>Environmental, premises, trespass</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -5406,12 +5389,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>nonprofit</t>
+          <t>other</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Nonprofit / social services</t>
+          <t>Something else</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -5419,41 +5402,9 @@
           <t>other</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Governance, volunteers, vulnerable clients</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>D&amp;O, abuse/molestation controls, professional liability</t>
-        </is>
-      </c>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
       <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Something else</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>

<commit_message>
Realign the diagnostic to the real estate vertical and tighten mobile layouts (#5)
Question bank, findings, checklist, niches, modules, producer brief,
industries, labels, schemas, and docs now target commercial real estate
owners and multifamily owners/managers, with real estate branch
triggers (owned buildings, third-party manager, site vendors,
residential tenants, workforce, investors, environmental). FMCSA
enrichment is removed. Reporting question columns are renamed for the
new industries. The public header, producer header, dashboard stats,
assessment form footers, and lead page grid are adjusted so nothing
overflows at phone widths; verified with screenshots at 390px and 1280px.


Claude-Session: https://claude.ai/code/session_01JbEPs9eRjvDhvYpso2k2wq

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/marketready-question-bank.xlsx
+++ b/docs/marketready-question-bank.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from code on 2026-09-02T19:38:39.475Z. Regenerate with: npm run docs:bank</t>
+          <t>Generated from code on 2026-09-02T21:30:54.262Z. Regenerate with: npm run docs:bank</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -587,7 +587,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -675,12 +675,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>business changes 0; profile recent change true/false</t>
+          <t>business changes 0; profile recent acquisition true/false</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -692,22 +692,22 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>fleet_branch</t>
+          <t>management_agreement_branch</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>hasVehicles true; fleet controls 0</t>
+          <t>usesThirdPartyManager true; management agreement 0</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>branch applicable; critical flag br_fleet_controls</t>
+          <t>branch applicable; critical flag br_management_agreement</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>module=contracts; COI 0, requirements 1, subcontractor 1</t>
+          <t>module=contracts; COI 0, requirements 1, vendor transfer 1</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Who owns the insurance program, when renewal work begins, and how limits are decided.</t>
+          <t>Who owns the insurance program across the portfolio, when renewal work begins, and how limits and deductibles are decided.</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Data &amp; market readiness</t>
+          <t>Property data &amp; market readiness</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>How well exposure data and business changes are documented and presented to carriers.</t>
+          <t>How well the statement of values, acquisitions and dispositions, and building updates are documented and presented to carriers.</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Cyber, payment authorization, safety, and training practices that underwriters ask about.</t>
+          <t>Tenant and applicant data, rent and vendor payment controls, and property inspection and life-safety practices.</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>How incidents are reported, open claims are reviewed, and root causes are tracked.</t>
+          <t>How incidents at the properties are reported, open claims are reviewed, and corrective actions are tracked.</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Whether contracts, insurance requirements, and certificate verification work as one system.</t>
+          <t>Whether leases, vendor agreements, insurance requirements, and certificate verification work as one system.</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>How new locations, products, technology, and regulations are reviewed for risk impact.</t>
+          <t>How acquisitions, new property types, regulations, and new exposures like EV charging are reviewed for risk impact.</t>
         </is>
       </c>
     </row>
@@ -1006,88 +1006,88 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>3PL, warehousing &amp; distribution</t>
+          <t>Commercial real estate owner / investor</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>3PL / Warehousing</t>
+          <t>Commercial RE</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Third-party logistics, public and contract warehousing, cold chain, fulfillment, and regional distribution.</t>
+          <t>Office, industrial and flex, retail, mixed-use, and net-lease portfolios, whether self-managed or with a third-party manager.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>493110, 493120, 484110, 484121, 488510</t>
+          <t>531110, 531120, 531190, 531390</t>
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Carriers evaluating warehousing and 3PL accounts look closely at warehouse legal liability, cargo and customer contracts, fleet controls, fire protection, and how consistently incidents are reported.</t>
+          <t>Property underwriters price commercial portfolios on the quality of the statement of values, construction and protection data, roof and building-system updates, how carrier recommendations were handled, and how lease and vendor requirements transfer risk.</t>
         </is>
       </c>
       <c r="H2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="I2" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="4" t="n">
         <v>1.25</v>
       </c>
-      <c r="J2" s="4" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="L2" s="4" t="n">
-        <v>1.5</v>
-      </c>
       <c r="M2" s="4" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Light manufacturing</t>
+          <t>Multifamily owner / property manager</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Multifamily</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Fabrication, assembly, food and beverage, plastics, packaging, electronics, and other light industrial operations.</t>
+          <t>Apartment communities, student and workforce housing, and third-party residential management.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>332, 333, 335, 311, 326, 339</t>
+          <t>531110, 531311, 531390</t>
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Underwriters reviewing manufacturers focus on product liability and recall exposure, machine guarding and workers' compensation history, property valuation, business interruption, and supplier and customer contract terms.</t>
+          <t>Multifamily carriers look closely at habitability and life-safety practices, renters insurance enforcement, fair-housing training, vendor certificates for snow and ice and contractors, claim frequency, and how quickly incidents are reported.</t>
         </is>
       </c>
       <c r="H3" s="4" t="n">
@@ -1103,7 +1103,7 @@
         <v>1.25</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="M3" s="4" t="n">
         <v>1</v>
@@ -1117,26 +1117,30 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Other middle-market business</t>
+          <t>Other real estate operator</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Other RE</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Any other commercial operation. Uses generic weighting.</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr"/>
+          <t>Self-storage, hospitality assets, senior housing, associations, land, or a mixed portfolio. Uses generic weighting.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
       <c r="F4" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Carriers evaluate every account on the quality of its exposure data, controls, claims history, and the clarity of the story that accompanies the submission.</t>
+          <t>Carriers evaluate every real estate account on the quality of its property data, the controls at each location, claims history, and the clarity of the story that accompanies the submission.</t>
         </is>
       </c>
       <c r="H4" s="4" t="n">
@@ -1224,12 +1228,12 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>weight_logistics_3pl</t>
+          <t>weight_cre_owner</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>weight_light_manufacturing</t>
+          <t>weight_multifamily</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
@@ -1270,12 +1274,12 @@
       <c r="E2" s="4" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>When does renewal preparation typically begin relative to your policy expiration?</t>
+          <t>When does renewal preparation for the portfolio typically begin relative to policy expiration?</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Carriers reward complete submissions delivered early. Late starts compress negotiation time.</t>
+          <t>Property markets reward complete, early submissions. A late start means values and building updates never make it into the story carriers see.</t>
         </is>
       </c>
       <c r="H2" s="4" t="n">
@@ -1292,7 +1296,7 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Renewal preparation appears to begin inside 30 days of expiration, which limits the ability to document controls and approach alternative markets.</t>
+          <t>Renewal preparation appears to begin inside 30 days of expiration, which limits the ability to update values, document building improvements, and approach alternative markets.</t>
         </is>
       </c>
     </row>
@@ -1318,10 +1322,14 @@
       <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Who owns the insurance program internally, and how is that responsibility defined?</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
+          <t>Who owns the insurance program for the portfolio, and how is that responsibility defined?</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>In many real estate organizations this sits between ownership, an asset manager, a controller, and the property manager.</t>
+        </is>
+      </c>
       <c r="H3" s="4" t="n">
         <v>2</v>
       </c>
@@ -1350,18 +1358,18 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Limit rationale</t>
+          <t>Limit and deductible rationale</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>How are policy limits and deductibles decided each year?</t>
+          <t>How are liability limits, property deductibles, and umbrella limits decided each year?</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>This question asks about your decision process, not whether the limits are adequate.</t>
+          <t>This asks about your decision process, not whether the limits are adequate.</t>
         </is>
       </c>
       <c r="H4" s="4" t="n">
@@ -1392,16 +1400,20 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Exposure data</t>
+          <t>Statement of values</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>How are exposure values (payroll, revenue, property values, vehicle schedules, inventory) validated before submission?</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr"/>
+          <t>How is the statement of values (replacement cost, construction and protection details, occupancy, square footage, year built, updates) maintained and validated before submission?</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Replacement cost that is dictated by the insurer, or carried forward, is the most common reason a property submission is discounted.</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="n">
         <v>3</v>
       </c>
@@ -1430,13 +1442,13 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Business change documentation</t>
+          <t>Portfolio changes</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>How are operational changes (new services, locations, equipment, customers, headcount) communicated to your insurance program during the year?</t>
+          <t>How are acquisitions, dispositions, renovations, new leases, and occupancy changes communicated to your insurance program during the year?</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -1468,18 +1480,18 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Submission visibility</t>
+          <t>Your risk profile in the market</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>How much visibility do you have into what is actually sent to carriers about your company?</t>
+          <t>Do you know how your story is being told in the marketplace, and do you see what is sent to insurance companies about the portfolio?</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>The underwriting story is the narrative and evidence that accompanies applications and loss runs.</t>
+          <t>Brokers who never saw your environmental consultant's report, your capital plan, or your maintenance program cannot present them.</t>
         </is>
       </c>
       <c r="H7" s="4" t="n">
@@ -1510,21 +1522,25 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Cyber controls</t>
+          <t>Data security</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr"/>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Which of the following best describes your cyber controls (MFA, backups, endpoint protection, incident response)?</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr"/>
+          <t>What data do you hold on tenants, applicants, and investors, how is it stored and shared, and how is it protected?</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Applications, background checks, banking details, and investor reporting are all sensitive. Property-management software vendors should be part of the answer.</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>2</v>
@@ -1534,7 +1550,7 @@
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Multi-factor authentication and tested backups do not appear to be consistently in place. Most cyber carriers now treat these as minimum requirements.</t>
+          <t>Tenant, applicant, or investor data appears to be held without a data security program. Cyber carriers treat MFA and encryption as minimum requirements.</t>
         </is>
       </c>
     </row>
@@ -1554,13 +1570,13 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Payment &amp; wire controls</t>
+          <t>Funds transfer security</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>How are changes to vendor bank details and outgoing wire requests verified?</t>
+          <t>How is the flow of funds controlled: rent collection, security deposits, vendor payments, wires, and changes to vendor bank details?</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
@@ -1578,7 +1594,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Vendor bank-detail changes and wires may be released on an email or phone request alone, which is the most common path for social-engineering losses.</t>
+          <t>Wires and vendor bank-detail changes may be released on an email or phone request alone, which is the most common path for social-engineering losses in property operations.</t>
         </is>
       </c>
     </row>
@@ -1598,16 +1614,20 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Safety &amp; training</t>
+          <t>Inspections, life safety &amp; maintenance</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>How are safety programs, training, and inspections documented?</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr"/>
+          <t>How are property inspections, life-safety systems, lighting, and preventive maintenance documented across the portfolio?</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Documented inspections and maintenance logs are what carriers credit; practices that exist only in the property manager's head do not count.</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="n">
         <v>3</v>
       </c>
@@ -1636,13 +1656,13 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Incident reporting</t>
+          <t>Claim intake &amp; reporting</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>What happens when an incident or potential claim occurs?</t>
+          <t>What policies and procedures make sure incidents at the properties (injuries, fires, water losses, tenant claims) are reported and managed properly?</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
@@ -1660,7 +1680,7 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Incidents appear to be reported inconsistently or late. Late reporting is a frequent driver of higher claim costs and coverage disputes.</t>
+          <t>Incidents appear to be reported inconsistently or late. Late reporting is a frequent driver of higher claim costs and coverage disputes, especially on liability claims.</t>
         </is>
       </c>
     </row>
@@ -1680,16 +1700,20 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Open claim review</t>
+          <t>Claims management &amp; advocacy</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>How often are open claims and reserves reviewed with your broker or carrier?</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
+          <t>How are open claims, reserves, carrier-assigned counsel, and public adjusters managed?</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>The workshop asks whether your broker has a systematic process: frequency of updates, claims positioning, policy review, legal guidance, and advocacy.</t>
+        </is>
+      </c>
       <c r="H12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1724,7 +1748,7 @@
       <c r="E13" s="4" t="inlineStr"/>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>After an incident, how are root causes identified and corrective actions tracked?</t>
+          <t>After an incident at a property, how are root causes identified and corrective actions tracked?</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
@@ -1756,21 +1780,21 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Signed contracts</t>
+          <t>Vendor &amp; contractor contracts</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Before work begins with customers, vendors, or subcontractors, how consistently are written contracts in place?</t>
+          <t>Tell us about the contracts you use with vendors and contractors at the properties (snow and ice, landscaping, security, renovations). Are master agreements in place with key vendors?</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr"/>
       <c r="H14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>2</v>
@@ -1794,13 +1818,13 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Insurance requirements</t>
+          <t>Insurance requirements in leases &amp; contracts</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>How do you determine what insurance to require from the parties you work with, and what they require from you?</t>
+          <t>How are insurance requirements set for tenants in leases and for vendors in contracts, and how are lender and management-agreement requirements on you tracked?</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
@@ -1832,13 +1856,13 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Certificate verification</t>
+          <t>Certificate tracking</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>How are certificates of insurance and endorsements (additional insured, waiver of subrogation) verified?</t>
+          <t>What is your process for vetting vendors and contractors who work at the properties, and how are certificates of insurance and endorsements tracked?</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -1846,7 +1870,7 @@
         <v>3</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>2</v>
@@ -1856,7 +1880,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Certificates of insurance are collected but not reviewed, so contractual risk transfer may not be operating when a loss occurs.</t>
+          <t>Vendor certificates of insurance are collected but not reviewed, so the indemnity and additional-insured protection in your contracts may not be operating when a loss occurs.</t>
         </is>
       </c>
     </row>
@@ -1876,18 +1900,18 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Annual risk review</t>
+          <t>Frequent risk assessment</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Does leadership conduct a structured risk review outside of the insurance renewal?</t>
+          <t>How often is a thorough risk assessment of the portfolio performed outside of an insurance policy renewal?</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>A risk review looks at operations, contracts, and controls, not just the policies being renewed.</t>
+          <t>A risk review looks at operations, contracts, properties, and controls, not just the policies being renewed.</t>
         </is>
       </c>
       <c r="H17" s="4" t="n">
@@ -1918,13 +1942,13 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Regulatory monitoring</t>
+          <t>Regulatory &amp; compliance monitoring</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>How are regulatory and compliance changes affecting your operations monitored?</t>
+          <t>How are regulatory and compliance changes affecting the properties monitored (fair housing, ADA, local habitability and safety ordinances, energy and benchmarking rules)?</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -1956,16 +1980,20 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>New activity review</t>
+          <t>New exposure review</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>When you add a new location, product, service, technology, or major customer, is risk and insurance impact reviewed beforehand?</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr"/>
+          <t>When you acquire a property, add a new property type, allow short-term rentals, or add EV charging or lithium-battery storage, is the risk and insurance impact reviewed beforehand?</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>The workshop found owners who had never heard of the lithium-battery exposure and were about to add car chargers.</t>
+        </is>
+      </c>
       <c r="H19" s="4" t="n">
         <v>2</v>
       </c>
@@ -1994,7 +2022,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Property valuation &amp; building updates</t>
+          <t>Carrier recommendations &amp; building updates</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2004,12 +2032,12 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>For the buildings you own, how are replacement values, business-interruption values, flood exposure, building updates (roof, sprinklers, electrical), and carrier loss-control recommendations documented and tracked?</t>
+          <t>What is your procedure for dealing with insurance company recommendations (sprinklers, wiring, boilers, roofs), and how are building updates and flood exposure documented?</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Carriers issue recommendations after inspections. How you respond to them is part of the underwriting story.</t>
+          <t>Carriers issue recommendations after inspections. Owners who track and close them, and show the carrier, negotiate from strength.</t>
         </is>
       </c>
       <c r="H20" s="4" t="n">
@@ -2030,27 +2058,27 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>operational_controls</t>
+          <t>contractual_risk_transfer</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Fleet &amp; driver controls</t>
+          <t>Management agreements</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>hasVehicles</t>
+          <t>usesThirdPartyManager</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>How are drivers screened and vehicles managed (MVRs, telematics, hired and non-owned auto)?</t>
+          <t>How do your management agreements address insurance and indemnification obligations between you and the third-party property manager?</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -2058,7 +2086,7 @@
         <v>3</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J21" s="4" t="n">
         <v>2</v>
@@ -2068,7 +2096,7 @@
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>Motor vehicle records do not appear to be run consistently, which commercial auto underwriters treat as a primary control.</t>
+          <t>Insurance and indemnification terms in the property-management agreement have not been reviewed, so it is unclear who is covered for a loss at a managed property.</t>
         </is>
       </c>
     </row>
@@ -2078,17 +2106,17 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>contractual_risk_transfer</t>
+          <t>operational_controls</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor &amp; vendor risk transfer</t>
+          <t>Snow &amp; ice, security, and site vendors</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -2098,15 +2126,15 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>For subcontractors and vendors, how consistently are indemnity terms, additional-insured status, and waivers of subrogation obtained and enforced?</t>
+          <t>For snow and ice removal, security patrols, and other on-site vendors, how consistently are procedures documented and risk transferred (logs, cameras, indemnity, additional-insured status)?</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
       <c r="H22" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>2</v>
@@ -2120,7 +2148,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2130,25 +2158,25 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Sensitive data handling</t>
+          <t>Leasing, renters insurance &amp; fair housing</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>storesSensitiveData</t>
+          <t>hasResidentialTenants</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>For the sensitive customer, employee, or payment data you hold, how are access, vendor security, and incident response managed?</t>
+          <t>For residential tenants, how are leasing and screening, renters-insurance verification, anti-discrimination training, and short-term-rental monitoring handled?</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
       <c r="H23" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J23" s="4" t="n">
         <v>2</v>
@@ -2182,12 +2210,12 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>With a workforce of this size, how are workers' compensation return-to-work, employment practices (handbook, training, documentation), and benefits data protection handled?</t>
+          <t>With on-site and corporate staff of this size, how are workers' compensation return-to-work, employment practices (handbook, training, documentation), and manager training handled?</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>
       <c r="H24" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I24" s="4" t="n">
         <v>3</v>
@@ -2214,7 +2242,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Board &amp; investor governance</t>
+          <t>Investors, funds &amp; lenders</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2224,12 +2252,12 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>With outside investors or a board, how are directors &amp; officers, fiduciary, and governance-related exposures reviewed?</t>
+          <t>With outside investors, funds, or lenders, how are investor reporting, fund and entity E&amp;O and D&amp;O exposures, and lender insurance requirements managed?</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr"/>
       <c r="H25" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>2</v>
@@ -2246,7 +2274,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2256,22 +2284,22 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Regulated materials &amp; environmental</t>
+          <t>Environmental risks</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>regulatedMaterials</t>
+          <t>environmentalExposures</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>For regulated materials or processes, how are environmental permits, storage practices, and pollution exposure managed?</t>
+          <t>What are your practices for environmental risks at the properties (lead, mold, asbestos, oil tanks, legionella, soil contamination), including due diligence on acquisitions?</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26" s="4" t="n">
         <v>3</v>
@@ -2344,7 +2372,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>About 60 days out, but it varies year to year</t>
+          <t>About 60 days out; we ask brokers to market and follow up 30 days out</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2387,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>90+ days out with a written timeline</t>
+          <t>90+ days out with a written timeline and an updated statement of values</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2402,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>120+ days out with a documented calendar, owners, and a pre-renewal strategy meeting</t>
+          <t>120+ days out with a documented calendar, owners, a pre-renewal strategy meeting, and a reconciled statement of values</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2417,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>No single owner; whoever the broker contacts handles it</t>
+          <t>No single owner; whoever the broker contacts handles it, or the property manager decides</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2447,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>A named owner with defined responsibilities</t>
+          <t>A named owner with defined responsibilities, including certificates and mid-term changes</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2462,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>A named owner, a backup, and a cross-functional review (finance, operations, HR/safety)</t>
+          <t>A named owner, a backup, and a defined split of duties with the property manager, asset management, and finance</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2477,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>We renew the same limits without discussion</t>
+          <t>We trust the agent or go with past numbers; limits follow the premium budget</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2492,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>The broker recommends and we generally accept</t>
+          <t>We have discussed limits with the agent but never worked through examples or lender requirements in detail</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2507,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>We review limits against contracts, assets, and revenue annually</t>
+          <t>We review limits annually against lender and lease requirements, asset values, and revenue</t>
         </is>
       </c>
     </row>
@@ -2494,7 +2522,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>We document the rationale for each limit and deductible and revisit it when the business changes</t>
+          <t>A formal annual process considers industry trends, risk tolerance, balance sheet, defensibility, lender covenants, and documents the rationale for each limit and deductible</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2537,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>We use last year's numbers unless someone flags a change</t>
+          <t>We don't analyze replacement cost; the insurer dictates it and values are carried forward</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2552,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>We update the big items but rarely reconcile schedules</t>
+          <t>We reviewed values a few years ago but do not update often and are not confident in the process</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2567,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Finance validates values annually against records</t>
+          <t>Values and building details are updated annually and checked against recent construction costs</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2582,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Values are reconciled against financials, fixed-asset registers, and schedules, with sign-off before submission</t>
+          <t>Values are updated annually, reconciled against rebuilds, appraisals, and recent claims, with construction, protection, and update history documented per building</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2612,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>We mention major changes when we remember</t>
+          <t>We mention major acquisitions or sales when we remember</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2627,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>A defined process captures changes and shares them with the broker</t>
+          <t>A defined process reports each acquisition, disposition, and major renovation to the broker with values and lender requirements</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2642,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Changes are logged, reviewed quarterly for insurance impact, and reflected in mid-term endorsements when needed</t>
+          <t>Changes are logged, reviewed quarterly for insurance impact, and reflected in schedules and endorsements when they happen</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2657,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>None; we sign applications and the broker handles the rest</t>
+          <t>I don't know; we have never seen what brokers present to market</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2672,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>We submit updated information annually but have not seen how our story is told to carriers</t>
+          <t>We submit updated information annually and confirm the broker understands changes to the portfolio</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2687,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>We review the submission and know which carriers quoted or declined</t>
+          <t>We review the submission and know which carriers quoted or declined and why</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2702,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>We collaborate with our broker on how best to portray the company in the marketplace, review the full submission, and receive a market summary with reasons for declinations</t>
+          <t>We collaborate with our broker to determine how best to portray the portfolio, review the full submission and narrative, and receive a market summary with reasons for declinations</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2717,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Basic antivirus; MFA and tested backups are not consistently in place</t>
+          <t>No data security program or process; information is stored locally and not encrypted</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2732,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>MFA on email; backups exist but are not tested regularly</t>
+          <t>Some form of data security, such as limited access, encryption, or occasional employee education</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2747,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>MFA on email and remote access, tested offline backups, endpoint detection, and a written incident plan</t>
+          <t>A formal data security program: MFA, encryption, limited access, regular training, and a written incident plan</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2762,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>All of the prior plus annual testing, vendor security review, and executive reporting</t>
+          <t>Formal program plus vendor security review of property-management and payment platforms, tested backups, and annual review with the broker</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2777,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>No formal protocol; an email or phone request is usually sufficient</t>
+          <t>No formal protocols; an email or phone request is usually sufficient</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2807,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Written procedure with callback verification to a known number and dual approval for all bank changes and wires</t>
+          <t>Written procedures with callback verification to a known number and dual approval for wires and bank-detail changes</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2822,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Formal written program with regular training: dual authorization, callback verification, destination confirmation, and receipt confirmation</t>
+          <t>Formal written program with regular training: dual authorization, calls to verify, destination-detail confirmation, receipt confirmation, and periodic consultation with the bank on best practices</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2837,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Training happens on the job; little is written down</t>
+          <t>Inspections happen when something breaks; little is written down</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2852,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Some written procedures; training records are incomplete</t>
+          <t>Some written procedures; inspection and maintenance records are incomplete or live only with the manager</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2867,7 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Written safety program, documented training, and periodic inspections</t>
+          <t>Written inspection schedule, life-safety testing records, and a preventive maintenance plan per property</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2882,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Written program with documented training, inspections, near-miss reporting, and management review of results</t>
+          <t>Written program with documented inspections, life-safety testing, lighting and security logs, preventive maintenance plans, and ownership review of results</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2897,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>It is reported when someone thinks of it, sometimes weeks later</t>
+          <t>No policies or protocols; the property manager reports claims directly to the carrier when they think of it</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2912,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Supervisors know to report, but timing and format vary</t>
+          <t>Supervisors and managers know to report, but timing and format vary; we check in with the broker when we need an update</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2927,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>A written protocol defines who reports, how, and within what timeframe</t>
+          <t>A written protocol defines who reports, how, and within what timeframe, with an incident form for every event</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2942,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Written protocol, reporting within 24–48 hours, an incident form, and tracking of every report</t>
+          <t>Written protocol, reporting within 24–48 hours, incident forms, and formal meetings with broker and adjusters on a predetermined timeline</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2957,7 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>We do not review open claims</t>
+          <t>We work directly with the carrier and adjuster; we do not focus on the liability claims process or communicate with assigned counsel</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2972,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Only when the carrier or broker raises something</t>
+          <t>We engage the broker if we are not satisfied; the broker primarily deals with counsel while we monitor open claims</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2987,7 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Scheduled reviews at least twice a year</t>
+          <t>Scheduled claim reviews at least twice a year with reserve discussion; we consider a public adjuster case by case</t>
         </is>
       </c>
     </row>
@@ -2974,7 +3002,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Quarterly claim reviews with reserve challenges, adjuster accountability, and pre-renewal loss-run reconciliation</t>
+          <t>A systematic process: quarterly reviews with reserve challenges, pre-assigned preferred defense counsel where possible, public-adjuster decisions made with the broker against policy wording, and pre-renewal loss-run reconciliation</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3032,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Supervisors discuss causes; actions are not tracked</t>
+          <t>The property manager discusses causes; actions are not tracked</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3047,7 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Root-cause review for significant incidents with documented corrective actions</t>
+          <t>Root-cause review for significant incidents with documented corrective actions and work orders</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3062,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Every incident gets a root-cause review, corrective actions are tracked to closure, and trends are reported to leadership</t>
+          <t>Every incident gets a root-cause review, corrective actions are tracked to closure across the portfolio, and trends are reported to ownership</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3077,7 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Often work starts on a handshake or PO alone</t>
+          <t>We don't always get contracts signed; work often starts on a proposal or a call</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3092,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Contracts exist for major relationships; smaller ones vary</t>
+          <t>An attorney reviews or writes contracts and we make sure they are signed</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3107,7 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Signed contracts are required before work begins</t>
+          <t>Attorney-reviewed contracts plus broker review for insurance and risk-transfer terms; signed before work starts</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3122,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Signed contracts required, with standard indemnity and insurance language reviewed by counsel and tracked centrally</t>
+          <t>Attorney and broker review, signed before work starts, master agreements with key vendors, and payment blocked when contract or insurance terms are missing</t>
         </is>
       </c>
     </row>
@@ -3109,7 +3137,7 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>We do not set requirements; we accept whatever the other party proposes</t>
+          <t>We do not set requirements; we accept whatever the tenant, vendor, or lender proposes</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3152,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>We use a generic requirement list without reviewing it</t>
+          <t>We use generic lease and contract language without reviewing it</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3167,7 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Requirements are defined by relationship type and reviewed by broker or counsel</t>
+          <t>Requirements are defined by relationship type (tenant, vendor, contractor) and reviewed by broker or counsel</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3182,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Requirements are defined, reviewed annually, and cross-checked against our own policies and customer demands</t>
+          <t>Requirements are defined, reviewed annually, cross-checked against our own policies and every lender and management-agreement obligation, and enforced</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3197,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>We collect certificates when asked but do not review them</t>
+          <t>We don't; certificates are collected when asked and not reviewed</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3212,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Someone checks that a certificate exists; endorsements are rarely verified</t>
+          <t>We obtain certificates with additional-insured status and check coverage and limit adequacy, but tracking is manual and infrequent</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3227,7 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Certificates and required endorsements are verified before work and on expiration</t>
+          <t>Certificates and required endorsements are verified before work and on expiration, in a tracking system</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3242,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Verification is tracked in a system, endorsements are matched to contract terms, and non-compliance is escalated</t>
+          <t>Software tracks every vendor's insurance in real time, the broker reviews complete policies for key contractors, endorsements are matched to contract terms, and non-compliant vendors are stopped from working</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3272,7 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>More than 18 months ago, or only when a new broker or agent first came on board</t>
+          <t>More than 18 months ago, or only when a new agent first came on board</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3287,7 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>An annual risk review with a documented risk list</t>
+          <t>Annually, with a documented list of risks by property</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3302,7 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Annual review with owners, action plans, and quarterly progress updates to leadership</t>
+          <t>Annually with owners and action plans, reviewed with the broker so prevention, mitigation, and insurance stay aligned</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3317,7 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>We learn about changes when we are notified of a violation or audit</t>
+          <t>We learn about changes when we are notified of a violation, complaint, or audit</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3347,7 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>A defined owner monitors regulations and briefs leadership</t>
+          <t>A defined owner monitors regulations, and required training and postings are documented</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3362,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Defined owner, documented compliance calendar, and periodic compliance audits</t>
+          <t>Defined owner, documented compliance calendar, annual training with records, and periodic compliance audits with counsel</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3392,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Sometimes, for very large changes</t>
+          <t>Sometimes, for very large acquisitions</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3407,7 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>A review step is included in the launch process</t>
+          <t>A review step with the broker is part of acquisition due diligence and major operational changes</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3422,7 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Documented pre-launch review with operations, finance, broker input, and follow-up after launch</t>
+          <t>Documented pre-acquisition and pre-launch review (environmental due diligence, valuation, lender requirements, new exposures) with follow-up after closing</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3437,7 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Values are carried forward; building updates and carrier recommendations are not tracked</t>
+          <t>We do as little as possible; updates and flood zones are not documented</t>
         </is>
       </c>
     </row>
@@ -3424,7 +3452,7 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Values were reviewed a few years ago; we do the minimum needed to stay compliant with carrier recommendations</t>
+          <t>We do the bare minimum to stay compliant with the insurer; updates are partially documented</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3467,7 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Replacement and BI values are reviewed annually; update history and recommendation responses are documented</t>
+          <t>An active protocol responds to and tracks recommendations; roof, sprinkler, electrical, and boiler updates are documented with dates</t>
         </is>
       </c>
     </row>
@@ -3454,14 +3482,14 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Professional valuation within three years, BI worksheet, flood zone determination, documented inspections and update history, and an active protocol for responding to and tracking every carrier recommendation</t>
+          <t>Active protocol for every recommendation with completion shown to the carrier, documented update history per building, flood zone determinations, and a professional valuation within three years</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="B78" s="4" t="n">
@@ -3469,14 +3497,14 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>We do not run MVRs consistently; personal vehicle use is not addressed</t>
+          <t>We do not review these requirements in agreements with our property managers</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="B79" s="4" t="n">
@@ -3484,14 +3512,14 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>MVRs at hire only; no written fleet policy</t>
+          <t>We accept the terms and conditions in the manager's boilerplate agreement</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="B80" s="4" t="n">
@@ -3499,14 +3527,14 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Written fleet policy, annual MVRs, and a defined hired/non-owned auto approach</t>
+          <t>Counsel reviewed the agreement; we know who insures what and hold the manager's certificate</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
       <c r="B81" s="4" t="n">
@@ -3514,14 +3542,14 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Written policy, annual MVRs with disqualification criteria, telematics or cameras, and driver training records</t>
+          <t>We actively review and dictate the insurance and indemnity terms, require adequate limits and coverages from the manager, and regularly request updated certificates to confirm they are in place</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="B82" s="4" t="n">
@@ -3529,14 +3557,14 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>We rely on the vendor's own paperwork</t>
+          <t>Employees or vendors handle it informally; no logs and contracts have not been reviewed</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="B83" s="4" t="n">
@@ -3544,14 +3572,14 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Our agreement includes the terms, but we rarely confirm the endorsements</t>
+          <t>Employees are trained or contractors are hired, but snow logs, security procedures, and contract terms are inconsistent</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="B84" s="4" t="n">
@@ -3559,14 +3587,14 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Terms are standard and endorsements are confirmed before work</t>
+          <t>Every snow removal and patrol is documented, and vendors indemnify and name us as additional insured</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
       <c r="B85" s="4" t="n">
@@ -3574,14 +3602,14 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Terms are standard, endorsements confirmed, non-compliant vendors are stopped from working, and exceptions are approved in writing</t>
+          <t>Documented logs visible on cameras, written security and snow procedures, contracts reviewed for indemnity and additional-insured terms, and vendor insurance tracked in a compliance system</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="B86" s="4" t="n">
@@ -3589,14 +3617,14 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Access is broad; we have not reviewed vendor security or an incident plan</t>
+          <t>No formal process; renters insurance is not tracked and fair-housing training is informal</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="B87" s="4" t="n">
@@ -3604,14 +3632,14 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Access is limited informally; incident response is undocumented</t>
+          <t>Application with employment verification and some screening; renters insurance tracked manually and updated infrequently; handbook statement only</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="B88" s="4" t="n">
@@ -3619,14 +3647,14 @@
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Role-based access, vendor security review, and a written incident response plan</t>
+          <t>Attorney-vetted application and lease, background checks, renters insurance required and tracked, annual fair-housing training, lease prohibits short-term rentals</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>br_data_security</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
       <c r="B89" s="4" t="n">
@@ -3634,7 +3662,7 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>All of the prior plus annual tabletop exercises, data inventory, and breach-notification readiness</t>
+          <t>All of the prior plus software that monitors renters insurance in real time and force-places when missing, documented annual training with counsel consultation, and active monitoring for short-term rental use</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3722,7 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>All of the prior plus experience-mod review, claims-trend analysis, and annual employment-practices training</t>
+          <t>All of the prior plus experience-mod review, claims-trend analysis, and annual employment-practices training with records</t>
         </is>
       </c>
     </row>
@@ -3709,7 +3737,7 @@
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>They have not been reviewed</t>
+          <t>Updates are provided on demand; entity coverages and lender requirements have not been reviewed</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3752,7 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Coverage was placed at the time of investment and not revisited</t>
+          <t>Annual performance updates; coverage was placed at the time of the raise and not revisited</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3767,7 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Reviewed annually with the broker against bylaws, investor agreements, and benefit plans</t>
+          <t>Quarterly reporting on performance and key metrics; E&amp;O and D&amp;O reviewed annually with the broker against fund documents; lender requirements tracked</t>
         </is>
       </c>
     </row>
@@ -3754,14 +3782,14 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Annual review plus board reporting on limits, indemnification agreements, and fiduciary controls</t>
+          <t>Quarterly reporting with online access, annual review of entity coverages, every legal entity confirmed as a named insured, and lender requirements reconciled at each closing</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="B98" s="4" t="n">
@@ -3769,14 +3797,14 @@
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>We are not sure what permits apply; storage practices are informal</t>
+          <t>I don't know; we have not looked at it</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="B99" s="4" t="n">
@@ -3784,14 +3812,14 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Permits are in place; documentation of storage and disposal is inconsistent</t>
+          <t>We depend on what we read and hear from industry groups; we may purchase environmental insurance</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="B100" s="4" t="n">
@@ -3799,14 +3827,14 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Permits, storage, and disposal are documented with a compliance owner</t>
+          <t>An environmental specialist has reviewed the portfolio and surveys; environmental due diligence is part of acquisitions</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_environmental</t>
         </is>
       </c>
       <c r="B101" s="4" t="n">
@@ -3814,7 +3842,7 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Documented compliance program, periodic environmental audits, and pollution exposure reviewed with the broker</t>
+          <t>Specialist reviews the portfolio routinely, moisture and mold procedures are written, lender environmental conditions are tracked, and environmental insurance is reviewed with the broker</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3868,31 +3896,35 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr"/>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>For a 3PL this includes the value of customers' goods in your care, custody, and control, vehicle and trailer schedules, and square footage by location.</t>
+          <t>Include unit counts, rent roll and business-income values, and any building improvements since the last valuation.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>mkt_exposure_data</t>
+          <t>ops_safety_training</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr"/>
+          <t>multifamily</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>How are unit and common-area inspections, life-safety systems (smoke and CO detectors, sprinklers, egress), lighting, and preventive maintenance documented across the communities?</t>
+        </is>
+      </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>For a manufacturer this includes machinery and equipment values, a business-interruption worksheet, and any dependence on a single supplier or customer.</t>
+          <t>Habitability claims turn on documentation: inspection logs, work-order completion, and life-safety testing records.</t>
         </is>
       </c>
     </row>
@@ -3904,157 +3936,73 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>How are warehouse and dock safety (forklift certification, racking, housekeeping), fire protection (sprinkler inspections, impairment procedures, commodity storage), and driver training documented?</t>
+          <t>How are roof, sprinkler, electrical, and boiler inspections, life-safety systems, and preventive maintenance documented across the buildings?</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Warehouse underwriters look first at fire protection and forklift and dock injury controls.</t>
+          <t>Roof age, sprinkler impairments, aluminum wiring, and boiler condition are the recommendations carriers issue most often.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>ops_safety_training</t>
+          <t>crt_insurance_requirements</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>How are machine guarding, lockout/tagout, hearing and respiratory protection, and safety training documented?</t>
-        </is>
-      </c>
+          <t>cre_owner</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Machine guarding and lockout/tagout drive both workers' compensation experience and product-safety credibility with underwriters.</t>
+          <t>Commercial leases typically require tenant liability and property coverage with the owner as additional insured; lenders require specific limits, mortgagee clauses, and flood where applicable.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>crt_signed_contracts</t>
+          <t>crt_insurance_requirements</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Before goods are received or work begins, how consistently are written warehousing agreements, customer contracts, and carrier/vendor agreements in place?</t>
-        </is>
-      </c>
+          <t>multifamily</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Warehouse receipts and customer contracts define your legal liability for goods in your care. Unsigned or inconsistent terms are a common gap.</t>
+          <t>Vendor requirements matter most here: snow and ice, security, and renovation contractors should indemnify and name the owner and manager as additional insureds.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>crt_signed_contracts</t>
+          <t>emr_regulatory</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>How consistently are written supply agreements, customer purchase terms, and vendor contracts in place before production or shipment begins?</t>
-        </is>
-      </c>
+          <t>multifamily</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Customer terms often carry product warranty, recall, and indemnity obligations that shape your liability program.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>crt_insurance_requirements</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>logistics_3pl</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Customers commonly require warehouse legal liability, cargo, and auto limits. Carriers and subcontracted haulers should be held to defined requirements in return.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>crt_insurance_requirements</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Large customers often specify product liability limits and vendor endorsements; suppliers should be held to defined requirements for the components they provide.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>emr_new_activity_review</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>logistics_3pl</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>When you take on a new commodity, temperature-controlled or hazardous storage, a new customer contract, or a new facility, is risk and insurance impact reviewed beforehand?</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>emr_new_activity_review</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>light_manufacturing</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>When you launch a new product, add a production line or process, or enter a new market, is product liability, recall, and business-interruption impact reviewed beforehand?</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr"/>
+          <t>Fair-housing training records, required postings, and consistent screening criteria are the first things asked about in a discrimination claim.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4067,7 +4015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4132,17 +4080,17 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Your renewal process may begin too late to fully document your risk controls.</t>
+          <t>Your renewal process may begin too late to fully document the portfolio.</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Renewal preparation appears to begin with limited runway. Controls that are not documented in time rarely make it into the submission carriers evaluate.</t>
+          <t>Renewal preparation appears to begin with limited runway. Updated values, building improvements, and closed carrier recommendations that are not documented in time rarely make it into the submission carriers evaluate.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Benchmark indication: high-impact underwriting strengths were identified elsewhere in your answers, but they may not be incorporated consistently into carrier submissions.</t>
+          <t>Benchmark indication: strengths were identified elsewhere in your answers, but they may not be incorporated consistently into what carriers see.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -4167,17 +4115,17 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Your contracts and insurance-verification process may not be operating as one control system.</t>
+          <t>Your leases, vendor contracts, and certificate tracking may not be operating as one control system.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Answers about signed contracts, insurance requirements, and certificate verification are uneven. Risk transfer only works when all three align.</t>
+          <t>Answers about signed vendor contracts, insurance requirements, and certificate verification are uneven. Risk transfer only works when the requirement, the contract, and the certificate line up.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: review whether contractual requirements, certificates of insurance, and policy endorsements align for your largest customer and vendor relationships.</t>
+          <t>Potential opportunity: review whether lease and contract requirements, certificates of insurance, and endorsements align for your largest tenants and your snow, security, and renovation vendors.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -4202,17 +4150,17 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Your business has changed faster than your insurance-governance process.</t>
+          <t>Your portfolio has changed faster than your insurance-governance process.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>You reported recent acquisitions or new locations, but operational changes reach the insurance program late or inconsistently.</t>
+          <t>You reported recent acquisitions, dispositions, or major renovations, but portfolio changes reach the insurance program late or inconsistently.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Areas to investigate: new locations, increased payroll, new services, and updated property values, and whether each is reflected in current schedules.</t>
+          <t>Areas to investigate: newly acquired properties, updated replacement values, lender requirements at each closing, and whether renovations are reflected in schedules.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -4242,12 +4190,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Incident reporting, open-claim review, or corrective-action tracking appear informal. Claims that are not managed tend to cost more and stay open longer.</t>
+          <t>Incident reporting, open-claim review, or corrective-action tracking appear informal, and there is no systematic broker process for advocacy, counsel, or public adjusters.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: evaluate reporting timelines, reserve review, adjuster accountability, and how corrective actions are tracked to closure.</t>
+          <t>Potential opportunity: evaluate reporting timelines, reserve review, carrier-assigned counsel, public-adjuster decisions, and how corrective actions are tracked across properties.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -4272,17 +4220,17 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Incomplete exposure data or a weak underwriting narrative could limit your market options.</t>
+          <t>A statement of values that carriers do not trust, or a story they never hear, could limit your market options.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Exposure values appear to be carried forward without reconciliation, or you have limited visibility into what carriers receive.</t>
+          <t>Replacement costs appear to be dictated by the insurer or carried forward, or you have limited visibility into what carriers receive about the portfolio.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Pricing cannot be assessed from this questionnaire alone. However, carriers generally offer their best terms to accounts that present validated data and a clear narrative, subject to policy, loss, and underwriting review.</t>
+          <t>Pricing cannot be assessed from this questionnaire alone. However, carriers generally offer their best terms to portfolios that present validated values, documented building updates, and a clear narrative, subject to policy, loss, and underwriting review.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -4307,17 +4255,17 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Payment-change and wire controls may leave a path open for social-engineering losses.</t>
+          <t>Funds-transfer controls may leave a path open for social-engineering losses.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Vendor bank-detail changes or wires may be released without callback verification and dual approval. This is the most common route for funds-transfer fraud.</t>
+          <t>Wires, vendor bank-detail changes, or security-deposit returns may be released without callback verification and dual approval. This is the most common route for funds-transfer fraud in property operations.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: confirm callback procedures, approval thresholds, and whether crime or cyber coverage includes social-engineering terms, subject to policy review.</t>
+          <t>Potential opportunity: confirm callback procedures, approval thresholds, controls at the property-management company, and whether crime or cyber coverage includes social-engineering terms, subject to policy review.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -4342,22 +4290,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Cyber controls may not meet the minimums that most carriers now require.</t>
+          <t>Protection of tenant, applicant, and investor data may not meet the minimums cyber carriers now require.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Multi-factor authentication, tested backups, and a written incident plan are the controls cyber underwriters ask about first.</t>
+          <t>Multi-factor authentication, encryption, tested backups, and a written incident plan are the controls cyber underwriters ask about first, along with the security of your property-management platform.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: document current controls, close gaps before the next cyber application, and confirm which controls are attested on existing applications.</t>
+          <t>Potential opportunity: document current controls, review the property-management and payment vendors' security, and confirm which controls are attested on existing applications.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>ops_cyber_controls, br_data_security</t>
+          <t>ops_cyber_controls</t>
         </is>
       </c>
     </row>
@@ -4377,17 +4325,17 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Insurance program ownership appears informal.</t>
+          <t>Insurance program ownership appears informal or split with the property manager.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Without a named owner and defined responsibilities, renewal tasks, certificate requests, and mid-term changes tend to fall through the cracks.</t>
+          <t>Without a named owner and a defined split of duties, certificate requests, mid-term acquisitions, and lender requirements tend to fall through the cracks.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: assign an owner and backup, and define the touchpoints with finance, operations, and HR/safety.</t>
+          <t>Potential opportunity: assign an owner and backup, and define who handles certificates, closings, and claims between ownership and the manager.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -4412,17 +4360,17 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Limits and deductibles appear to be renewed without a documented rationale.</t>
+          <t>Limits and deductibles appear to follow the budget rather than a documented rationale.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>This diagnostic does not assess whether limits are adequate. It does note that limits which are never revisited may not track contract requirements or asset growth.</t>
+          <t>This diagnostic does not assess whether limits are adequate. It does note that limits which are never revisited may not track lender covenants, lease requirements, or portfolio growth.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: document the basis for each limit and deductible with a licensed advisor and revisit it when contracts or assets change.</t>
+          <t>Potential opportunity: document the basis for each limit and deductible with a licensed advisor, including key liability cases and lender requirements, and revisit it as the portfolio changes.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -4447,17 +4395,17 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Safety and training practices may exist but are not documented in a form underwriters can credit.</t>
+          <t>Inspection, life-safety, and maintenance practices may exist but are not documented in a form underwriters can credit.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Written programs, training records, and inspection logs are what carriers use to distinguish a well-run operation from an average one.</t>
+          <t>Inspection schedules, life-safety testing records, lighting logs, and preventive maintenance plans are what carriers use to distinguish a well-run portfolio from an average one.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: assemble a safety documentation package before the next submission.</t>
+          <t>Potential opportunity: assemble an inspection and maintenance documentation package per property before the next submission.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -4478,21 +4426,21 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Owned-property values and building updates may be undocumented.</t>
+          <t>Carrier recommendations and building updates may not be tracked or shown to the market.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Replacement cost, business-interruption values, flood exposure, and building-system updates drive both coverage terms and pricing conversations.</t>
+          <t>How you respond to sprinkler, wiring, boiler, and roof recommendations, and whether updates and flood exposure are documented, drives both coverage terms and pricing conversations.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Areas to investigate: date of last valuation, BI worksheet, flood zone determination, and documented roof, sprinkler, and electrical updates.</t>
+          <t>Areas to investigate: open recommendations by property, completion evidence, roof and system update dates, flood zone determinations, and the date of the last professional valuation.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -4504,47 +4452,47 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>fleet_controls</t>
+          <t>management_agreement_gap</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>operational_controls</t>
+          <t>contractual_risk_transfer</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Fleet and driver controls may not be documented to the level auto underwriters expect.</t>
+          <t>The insurance and indemnity terms in your property-management agreement may not have been reviewed.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>MVR practices, fleet policy, and hired/non-owned auto handling are primary controls for commercial auto.</t>
+          <t>Boilerplate management agreements often leave it unclear who insures what and who indemnifies whom when a loss occurs at a managed property.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: adopt a written fleet policy with annual MVRs and disqualification criteria.</t>
+          <t>Potential opportunity: have counsel and the broker review the agreement, dictate required limits and coverages, and hold current certificates from the manager.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>br_fleet_controls</t>
+          <t>br_management_agreement</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>subcontractor_transfer_gap</t>
+          <t>site_vendor_gap</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>contractual_risk_transfer</t>
+          <t>operational_controls</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -4552,29 +4500,29 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor and vendor risk transfer may not be enforced.</t>
+          <t>Snow and ice, security, and site-vendor procedures may not be documented or transferring risk.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Indemnity terms and endorsements that are not confirmed before work begins may not respond when a loss occurs.</t>
+          <t>Slip-and-fall and premises claims turn on logs, cameras, and whether the vendor's contract indemnifies and insures you.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: confirm additional-insured and waiver endorsements for active vendors.</t>
+          <t>Potential opportunity: require documented snow logs and patrol procedures, and confirm indemnity and additional-insured terms for every site vendor.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>br_subcontractor_transfer</t>
+          <t>br_vendor_transfer</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>workforce_programs_gap</t>
+          <t>residential_programs_gap</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -4583,129 +4531,164 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Workforce programs (return-to-work, handbook, manager training) may be informal for a company of your size.</t>
+          <t>Leasing, renters-insurance, and fair-housing practices may be informal for the size of the residential portfolio.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>These programs influence workers' compensation experience and employment-practices exposure.</t>
+          <t>Renters insurance that is not tracked, screening that is not consistent, and training that is not documented all show up in liability and discrimination claims.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: document return-to-work procedures and update the employee handbook.</t>
+          <t>Potential opportunity: evaluate real-time renters-insurance monitoring, attorney-vetted lease and screening criteria, and documented annual fair-housing training.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>br_workforce_programs</t>
+          <t>br_residential_programs</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>investor_governance_gap</t>
+          <t>workforce_programs_gap</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>operational_controls</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Board and investor-related exposures may not have been reviewed since the investment.</t>
+          <t>Workforce programs (return-to-work, handbook, manager training) may be informal for a staff of your size.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Directors &amp; officers, fiduciary, and indemnification arrangements are typically revisited as ownership and boards change.</t>
+          <t>These programs influence workers' compensation experience and employment-practices exposure across on-site teams.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Potential opportunity: review governance-related exposures with a licensed advisor against current bylaws and investor agreements.</t>
+          <t>Potential opportunity: document return-to-work procedures and update the employee handbook.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>br_governance_investors</t>
+          <t>br_workforce_programs</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>environmental_gap</t>
+          <t>investor_governance_gap</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>emerging_risk</t>
+          <t>governance</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Environmental compliance and pollution exposure may not be documented.</t>
+          <t>Investor, fund, and lender-related exposures may not have been reviewed since the last capital event.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Permits, storage practices, and disposal records are the starting point for any environmental conversation with carriers.</t>
+          <t>Fund and entity E&amp;O and D&amp;O, named-insured completeness across every LLC, and lender requirements are typically revisited as deals close and boards change.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Areas to investigate: applicable permits, storage documentation, and whether pollution exposure has been reviewed.</t>
+          <t>Potential opportunity: review entity coverages with a licensed advisor against fund documents and confirm every legal entity is scheduled as a named insured.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>br_regulated_materials</t>
+          <t>br_governance_investors</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>environmental_gap</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>emerging_risk</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Environmental exposures at the properties may not have been reviewed.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Lead, mold, asbestos, oil tanks, legionella, and soil conditions are the starting point for any environmental conversation with carriers and lenders.</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Areas to investigate: environmental surveys on file, acquisition due diligence, moisture and mold procedures, lender environmental conditions, and whether pollution exposure has been reviewed.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>br_environmental</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>emerging_risk_unmanaged</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>emerging_risk</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C19" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>New activities and regulatory changes may reach the insurance program after the fact.</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Without a pre-launch review step, new locations, products, and technology can create exposures that are not reflected until the next renewal.</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Potential opportunity: add a risk and insurance checkpoint to your launch process.</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Acquisitions, regulatory changes, and new exposures may reach the insurance program after the fact.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Without a pre-acquisition and pre-launch review step, new properties, short-term rentals, EV charging, and lithium-battery storage can create exposures that are not reflected until the next renewal.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Potential opportunity: add a risk and insurance checkpoint to acquisition due diligence and to operational changes at the properties.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>emr_new_activity_review, emr_regulatory, emr_annual_review</t>
         </is>
@@ -4790,7 +4773,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>How ready is your company to be evaluated by the insurance market?</t>
+          <t>How ready is your real estate portfolio to be evaluated by the insurance market?</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -4800,7 +4783,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>CFOs, COOs, and owners unsure whether the company is presenting an accurate, differentiated risk story.</t>
+          <t>Owners, asset managers, and CFOs unsure whether the portfolio is presenting an accurate, differentiated risk story.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr"/>
@@ -4820,17 +4803,17 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Is your next renewal on a timeline, or on autopilot?</t>
+          <t>Is your property renewal on a timeline, or on autopilot?</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>A confidential check of your renewal runway, the data carriers will ask for, and the changes that need to be documented before submissions go out.</t>
+          <t>A confidential check of your renewal runway, the statement of values carriers will scrutinize, and the acquisitions and updates that need to be documented before submissions go out.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>CFOs and risk managers facing a renewal within three to nine months.</t>
+          <t>Owners, asset managers, and CFOs facing a property renewal within three to nine months.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -4845,7 +4828,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Timing, data, and the story carriers receive. These answers determine whether preparation starts early enough to matter.</t>
+          <t>Timing, values, and the story carriers receive. These answers determine whether preparation starts early enough to matter.</t>
         </is>
       </c>
     </row>
@@ -4862,17 +4845,17 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Are your contracts actually transferring risk, or just describing it?</t>
+          <t>Are your leases and vendor contracts actually transferring risk, or just describing it?</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>A confidential scan of how signed contracts, insurance requirements, certificates, and subcontractor terms work together as one control system.</t>
+          <t>A confidential scan of how leases, vendor and snow-removal contracts, management agreements, insurance requirements, and certificate tracking work together as one control system.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>COOs and CFOs in construction, manufacturing, real estate, and logistics who rely on vendors and subcontractors.</t>
+          <t>Owners and property managers who rely on tenants' insurance and on-site vendors.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -4882,12 +4865,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Your contract-risk workflow</t>
+          <t>Your lease and vendor risk-transfer workflow</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Requirements that are never verified, and certificates that are never matched to contracts, do not transfer risk when a loss occurs.</t>
+          <t>Requirements that are never verified, and certificates that are never matched to leases and contracts, do not transfer risk when a loss occurs.</t>
         </is>
       </c>
     </row>
@@ -4904,17 +4887,17 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Are claims being managed, or just reported?</t>
+          <t>Are claims at your properties being managed, or just reported?</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>A confidential look at reporting speed, open-claim cadence, return-to-work practices, and how corrective actions are tracked.</t>
+          <t>A confidential look at reporting speed, open-claim cadence, public-adjuster and counsel practices, and how corrective actions are tracked across the portfolio.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>CFO, HR, and operations leaders frustrated by recurring or poorly managed claims.</t>
+          <t>Owners, asset managers, and property managers frustrated by recurring or poorly managed claims.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -4929,7 +4912,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Late reporting, unreviewed reserves, and untracked corrective actions are the most common reasons claims cost more and stay open longer.</t>
+          <t>Late reporting, unreviewed reserves, unmanaged counsel, and untracked corrective actions are the most common reasons property claims cost more and stay open longer.</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4990,27 +4973,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>3PL / warehousing / distribution</t>
+          <t>Multifamily / apartment communities</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Fleet, property, cargo, labor, contracts</t>
+          <t>Tenant, premises, discrimination</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Cargo, auto, warehouse legal liability, fire protection</t>
+          <t>Renters insurance, habitability, EPLI, vendor controls</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -5022,59 +5005,59 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>food_cold_storage</t>
+          <t>office</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Food distribution / cold storage</t>
+          <t>Office</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>logistics_3pl</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Spoilage and temperature dependency</t>
+          <t>Property values and tenant improvements</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Refrigeration breakdown, recall, contamination</t>
+          <t>SOV quality, lease requirements, BI, life safety</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>industrial_flex</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Light / advanced manufacturing</t>
+          <t>Industrial / flex / warehouse</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Property, machinery, products, WC</t>
+          <t>Large replacement values and tenant operations</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Business interruption, machine guarding, product liability</t>
+          <t>SOV quality, sprinkler and roof condition, tenant contracts, environmental</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -5086,76 +5069,76 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>life_sciences</t>
+          <t>retail_mixed_use</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Life-sciences supplier</t>
+          <t>Retail / mixed-use</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>light_manufacturing</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>High-value inventory and regulated work</t>
+          <t>Premises liability and vendor dependence</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Clinical/product liability, cold chain, cyber, E&amp;O</t>
+          <t>Snow and ice, security, lease requirements, liquor tenants</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>contractors</t>
+          <t>net_lease</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Contractor / trades</t>
+          <t>Net-lease / single-tenant</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Subcontracting and contractual risk</t>
+          <t>Lease-driven insurance obligations</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Wrap-ups, fleet, jobsite safety, certificates</t>
+          <t>Tenant compliance tracking, lender requirements, named insureds</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>cre_owners</t>
+          <t>self_storage</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Commercial real estate owner</t>
+          <t>Self-storage</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -5165,12 +5148,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Property values and vendor dependence</t>
+          <t>Property, customer goods, access control</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>SOV quality, flood, BI, leases, management agreements</t>
+          <t>Customer goods legal liability, security, tenant insurance programs</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -5182,12 +5165,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>multifamily</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Multifamily / property manager</t>
+          <t>Hospitality / hotel assets</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -5197,12 +5180,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Tenant, premises, discrimination</t>
+          <t>Property, liquor, events, seasonal labor</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Renters insurance, habitability, EPLI, vendor controls</t>
+          <t>Liquor, pools, events, management agreements, D&amp;O</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -5214,12 +5197,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>healthcare</t>
+          <t>senior_housing</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Healthcare practice / MSO</t>
+          <t>Senior housing / assisted living</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -5229,12 +5212,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Professional, privacy, employment</t>
+          <t>Severe liability and workforce exposure</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Medical professional, cyber, regulatory, credentialing</t>
+          <t>Abuse controls, professional liability, staffing, auto</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -5246,44 +5229,44 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>senior_living</t>
+          <t>student_housing</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Senior living / home care</t>
+          <t>Student housing</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Severe liability and workforce exposure</t>
+          <t>Turnover, premises, parental guarantees</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Abuse controls, auto, professional liability, staffing</t>
+          <t>Renters insurance, security, event and alcohol exposure</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>professional_services</t>
+          <t>association</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Professional services</t>
+          <t>Condo / HOA association</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -5293,12 +5276,12 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>E&amp;O, cyber, executive risk</t>
+          <t>Governance, common areas, D&amp;O</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Contract scope, client concentration, privacy</t>
+          <t>D&amp;O, master policy allocation, vendor controls, reserves</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -5310,76 +5293,76 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>technology_msp</t>
+          <t>third_party_manager</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Technology / MSP</t>
+          <t>Third-party property manager</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>multifamily</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Contractual and cyber aggregation</t>
+          <t>Management-agreement exposure across many owners</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Tech E&amp;O, ransomware, dependent business interruption</t>
+          <t>Management agreements, E&amp;O, tenant discrimination, funds handling</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>auto_dealers</t>
+          <t>developer</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Auto dealer / fleet business</t>
+          <t>Developer / owner-builder</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cre_owner</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Inventory, garage, drivers</t>
+          <t>Construction and lease-up risk</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Garage liability, false pretense, cyber, weather</t>
+          <t>Builders risk, wrap-ups, contractor certificates, lender requirements</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>hospitality_clubs</t>
+          <t>land</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Hospitality / country club</t>
+          <t>Land / agricultural holdings</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -5389,12 +5372,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Property, liquor, events, seasonal labor</t>
+          <t>Premises and environmental</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Liquor, golf carts, pools, events, D&amp;O</t>
+          <t>Environmental, premises, trespass</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -5406,12 +5389,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>nonprofit</t>
+          <t>other</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Nonprofit / social services</t>
+          <t>Something else</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -5419,41 +5402,9 @@
           <t>other</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Governance, volunteers, vulnerable clients</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>D&amp;O, abuse/molestation controls, professional liability</t>
-        </is>
-      </c>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
       <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Something else</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>